<commit_message>
Rename project and refresh finalized viewer bundle
</commit_message>
<xml_diff>
--- a/data/finalized/curation/brain_mri_curation.xlsx
+++ b/data/finalized/curation/brain_mri_curation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rcf11e06b23b8491c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="Re83d82dbc67e42c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="R883d6835741d4ba2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Ra479c853f883412b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="Rc641740975034ecc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="Rf4b308503cb049bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -622,7 +622,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Brain MRI Curation Workbook</x:v>
+        <x:v>Neuroradiology Quizzer Curation Workbook</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -2006,7 +2006,7 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G43" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H43" s="35" t="str">
         <x:v>needs_review</x:v>
@@ -2418,7 +2418,7 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G57" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H57" s="35" t="str">
         <x:v>needs_review</x:v>
@@ -3167,17 +3167,11 @@
         <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F82" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G82" s="35" t="str">
-        <x:v>rough_support</x:v>
-      </x:c>
-      <x:c r="H82" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I82" s="35" t="str">
-        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G82" s="35" t="str"/>
+      <x:c r="H82" s="35" t="str"/>
+      <x:c r="I82" s="35" t="str"/>
       <x:c r="J82" s="35" t="str"/>
       <x:c r="K82" s="35" t="str"/>
       <x:c r="L82" s="36" t="str"/>
@@ -3292,7 +3286,7 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G86" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H86" s="35" t="str">
         <x:v>needs_review</x:v>
@@ -3568,10 +3562,10 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G95" s="35" t="str">
-        <x:v>rough_support</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H95" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I95" s="35" t="str">
         <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
@@ -3649,7 +3643,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c6c8b36a7c8474f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7763c544aa5c4f24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5925,7 +5919,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c1f6307b5e94c2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68dade5eaf1f484b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update viewer difficulty levels
</commit_message>
<xml_diff>
--- a/data/finalized/curation/brain_mri_curation.xlsx
+++ b/data/finalized/curation/brain_mri_curation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/siddhantdogra/Documents/Codex/Annotated Brain MRI/data/finalized/curation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F5A906C-B5D8-B74A-BB93-7921AD4ECE2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6B2D7C0-99C5-EB4F-AD54-49E95EEF6F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1697,7 +1697,7 @@
         <v>26</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>33</v>
@@ -1941,7 +1941,7 @@
         <v>26</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>65</v>
@@ -2025,7 +2025,7 @@
         <v>26</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>78</v>
@@ -2051,7 +2051,7 @@
         <v>26</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>81</v>
@@ -2675,7 +2675,7 @@
         <v>26</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>147</v>
@@ -2817,7 +2817,7 @@
         <v>26</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>162</v>
@@ -2939,7 +2939,7 @@
         <v>26</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>176</v>
@@ -3113,7 +3113,7 @@
         <v>26</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>194</v>
@@ -3261,7 +3261,7 @@
         <v>26</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>211</v>
@@ -3485,7 +3485,7 @@
         <v>26</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>234</v>
@@ -3569,7 +3569,7 @@
         <v>26</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>241</v>
@@ -3659,7 +3659,7 @@
         <v>26</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>250</v>
@@ -3685,7 +3685,7 @@
         <v>26</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>252</v>
@@ -3749,7 +3749,7 @@
         <v>26</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>257</v>
@@ -3775,7 +3775,7 @@
         <v>26</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>259</v>
@@ -3833,7 +3833,7 @@
         <v>26</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>264</v>
@@ -4007,7 +4007,7 @@
         <v>26</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>283</v>
@@ -4065,7 +4065,7 @@
         <v>26</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>290</v>
@@ -4129,7 +4129,7 @@
         <v>26</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>297</v>

</xml_diff>

<commit_message>
Add optic nerve target
</commit_message>
<xml_diff>
--- a/data/finalized/curation/brain_mri_curation.xlsx
+++ b/data/finalized/curation/brain_mri_curation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R3da4b9f4d05e43b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="R4827bd631bd04071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="R9224fb53500b4385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R362281277f0d48dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="R46e86ae690d14965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="R1e98051f2815417c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -375,7 +375,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StructureCurationTable" displayName="StructureCurationTable" ref="A1:L105" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StructureCurationTable" displayName="StructureCurationTable" ref="A1:L106" headerRowCount="1">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="include_in_viewer"/>
     <x:tableColumn id="2" name="difficulty"/>
@@ -395,7 +395,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuizQuestionTable" displayName="QuizQuestionTable" ref="A1:M105" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuizQuestionTable" displayName="QuizQuestionTable" ref="A1:M106" headerRowCount="1">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="display_name"/>
@@ -721,7 +721,7 @@
         <x:v>Structure count</x:v>
       </x:c>
       <x:c r="B9" s="5" t="n">
-        <x:v>104</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str"/>
       <x:c r="D9" s="5" t="str"/>
@@ -1146,7 +1146,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B14" s="34" t="str">
         <x:v>beginner</x:v>
@@ -1174,7 +1174,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B15" s="34" t="str">
         <x:v>beginner</x:v>
@@ -1992,7 +1992,7 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B43" s="34" t="str">
         <x:v>beginner</x:v>
@@ -2721,32 +2721,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B68" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C68" s="35" t="str">
-        <x:v>orbitofrontal_cortex</x:v>
+        <x:v>optic_nerve</x:v>
       </x:c>
       <x:c r="D68" s="35" t="str">
-        <x:v>Orbitofrontal cortex</x:v>
+        <x:v>Optic nerve</x:v>
       </x:c>
       <x:c r="E68" s="35" t="str">
-        <x:v>cortex; skull_base</x:v>
+        <x:v>cranial_nerves; skull_base; orbit</x:v>
       </x:c>
       <x:c r="F68" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G68" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H68" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I68" s="35" t="str">
-        <x:v>annotations/090_orbitofrontal_cortex.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G68" s="35" t="str"/>
+      <x:c r="H68" s="35" t="str"/>
+      <x:c r="I68" s="35" t="str"/>
       <x:c r="J68" s="35" t="str"/>
       <x:c r="K68" s="35" t="str"/>
-      <x:c r="L68" s="36" t="str"/>
+      <x:c r="L68" s="36" t="str">
+        <x:v>High-yield anterior skull base/orbital apex structure adjacent to the optic chiasm.</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="33" t="str">
@@ -2756,13 +2752,13 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C69" s="35" t="str">
-        <x:v>parahippocampal_gyrus</x:v>
+        <x:v>orbitofrontal_cortex</x:v>
       </x:c>
       <x:c r="D69" s="35" t="str">
-        <x:v>Parahippocampal gyrus</x:v>
+        <x:v>Orbitofrontal cortex</x:v>
       </x:c>
       <x:c r="E69" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex; skull_base</x:v>
       </x:c>
       <x:c r="F69" s="35" t="str">
         <x:v>yes</x:v>
@@ -2774,7 +2770,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I69" s="35" t="str">
-        <x:v>annotations/089_parahippocampal_gyrus.nii.gz</x:v>
+        <x:v>annotations/090_orbitofrontal_cortex.nii.gz</x:v>
       </x:c>
       <x:c r="J69" s="35" t="str"/>
       <x:c r="K69" s="35" t="str"/>
@@ -2785,60 +2781,60 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B70" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C70" s="35" t="str">
-        <x:v>parietal_lobe</x:v>
+        <x:v>parahippocampal_gyrus</x:v>
       </x:c>
       <x:c r="D70" s="35" t="str">
-        <x:v>Parietal lobe</x:v>
+        <x:v>Parahippocampal gyrus</x:v>
       </x:c>
       <x:c r="E70" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="F70" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G70" s="35" t="str"/>
-      <x:c r="H70" s="35" t="str"/>
-      <x:c r="I70" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G70" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H70" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I70" s="35" t="str">
+        <x:v>annotations/089_parahippocampal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J70" s="35" t="str"/>
       <x:c r="K70" s="35" t="str"/>
-      <x:c r="L70" s="36" t="str">
-        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
-      </x:c>
+      <x:c r="L70" s="36" t="str"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B71" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C71" s="35" t="str">
-        <x:v>parieto_occipital_sulcus</x:v>
+        <x:v>parietal_lobe</x:v>
       </x:c>
       <x:c r="D71" s="35" t="str">
-        <x:v>Parieto-occipital sulcus</x:v>
+        <x:v>Parietal lobe</x:v>
       </x:c>
       <x:c r="E71" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="F71" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G71" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H71" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I71" s="35" t="str">
-        <x:v>annotations/092_parieto_occipital_sulcus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G71" s="35" t="str"/>
+      <x:c r="H71" s="35" t="str"/>
+      <x:c r="I71" s="35" t="str"/>
       <x:c r="J71" s="35" t="str"/>
       <x:c r="K71" s="35" t="str"/>
-      <x:c r="L71" s="36" t="str"/>
+      <x:c r="L71" s="36" t="str">
+        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
+      </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="33" t="str">
@@ -2848,10 +2844,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C72" s="35" t="str">
-        <x:v>pars_opercularis</x:v>
+        <x:v>parieto_occipital_sulcus</x:v>
       </x:c>
       <x:c r="D72" s="35" t="str">
-        <x:v>Pars opercularis</x:v>
+        <x:v>Parieto-occipital sulcus</x:v>
       </x:c>
       <x:c r="E72" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2860,13 +2856,13 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G72" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H72" s="35" t="str">
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I72" s="35" t="str">
-        <x:v>annotations/017_pars_opercularis.nii.gz</x:v>
+        <x:v>annotations/092_parieto_occipital_sulcus.nii.gz</x:v>
       </x:c>
       <x:c r="J72" s="35" t="str"/>
       <x:c r="K72" s="35" t="str"/>
@@ -2880,10 +2876,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C73" s="35" t="str">
-        <x:v>pars_orbitalis</x:v>
+        <x:v>pars_opercularis</x:v>
       </x:c>
       <x:c r="D73" s="35" t="str">
-        <x:v>Pars orbitalis</x:v>
+        <x:v>Pars opercularis</x:v>
       </x:c>
       <x:c r="E73" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2898,7 +2894,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I73" s="35" t="str">
-        <x:v>annotations/018_pars_orbitalis.nii.gz</x:v>
+        <x:v>annotations/017_pars_opercularis.nii.gz</x:v>
       </x:c>
       <x:c r="J73" s="35" t="str"/>
       <x:c r="K73" s="35" t="str"/>
@@ -2912,10 +2908,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C74" s="35" t="str">
-        <x:v>pars_triangularis</x:v>
+        <x:v>pars_orbitalis</x:v>
       </x:c>
       <x:c r="D74" s="35" t="str">
-        <x:v>Pars triangularis</x:v>
+        <x:v>Pars orbitalis</x:v>
       </x:c>
       <x:c r="E74" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2930,7 +2926,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I74" s="35" t="str">
-        <x:v>annotations/019_pars_triangularis.nii.gz</x:v>
+        <x:v>annotations/018_pars_orbitalis.nii.gz</x:v>
       </x:c>
       <x:c r="J74" s="35" t="str"/>
       <x:c r="K74" s="35" t="str"/>
@@ -2941,23 +2937,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B75" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C75" s="35" t="str">
-        <x:v>pineal_gland</x:v>
+        <x:v>pars_triangularis</x:v>
       </x:c>
       <x:c r="D75" s="35" t="str">
-        <x:v>Pineal gland</x:v>
+        <x:v>Pars triangularis</x:v>
       </x:c>
       <x:c r="E75" s="35" t="str">
-        <x:v>midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F75" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G75" s="35" t="str"/>
-      <x:c r="H75" s="35" t="str"/>
-      <x:c r="I75" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G75" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H75" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I75" s="35" t="str">
+        <x:v>annotations/019_pars_triangularis.nii.gz</x:v>
+      </x:c>
       <x:c r="J75" s="35" t="str"/>
       <x:c r="K75" s="35" t="str"/>
       <x:c r="L75" s="36" t="str"/>
@@ -2970,13 +2972,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C76" s="35" t="str">
-        <x:v>pituitary_fossa</x:v>
+        <x:v>pineal_gland</x:v>
       </x:c>
       <x:c r="D76" s="35" t="str">
-        <x:v>Pituitary fossa</x:v>
+        <x:v>Pineal gland</x:v>
       </x:c>
       <x:c r="E76" s="35" t="str">
-        <x:v>skull_base; midline</x:v>
+        <x:v>midline</x:v>
       </x:c>
       <x:c r="F76" s="35" t="str">
         <x:v>no</x:v>
@@ -2996,26 +2998,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C77" s="35" t="str">
-        <x:v>pons</x:v>
+        <x:v>pituitary_fossa</x:v>
       </x:c>
       <x:c r="D77" s="35" t="str">
-        <x:v>Pons</x:v>
+        <x:v>Pituitary fossa</x:v>
       </x:c>
       <x:c r="E77" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>skull_base; midline</x:v>
       </x:c>
       <x:c r="F77" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G77" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H77" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I77" s="35" t="str">
-        <x:v>annotations/040_pons.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G77" s="35" t="str"/>
+      <x:c r="H77" s="35" t="str"/>
+      <x:c r="I77" s="35" t="str"/>
       <x:c r="J77" s="35" t="str"/>
       <x:c r="K77" s="35" t="str"/>
       <x:c r="L77" s="36" t="str"/>
@@ -3028,25 +3024,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C78" s="35" t="str">
-        <x:v>postcentral_gyrus</x:v>
+        <x:v>pons</x:v>
       </x:c>
       <x:c r="D78" s="35" t="str">
-        <x:v>Postcentral gyrus</x:v>
+        <x:v>Pons</x:v>
       </x:c>
       <x:c r="E78" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="F78" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G78" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H78" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I78" s="35" t="str">
-        <x:v>annotations/020_postcentral_gyrus.nii.gz</x:v>
+        <x:v>annotations/040_pons.nii.gz</x:v>
       </x:c>
       <x:c r="J78" s="35" t="str"/>
       <x:c r="K78" s="35" t="str"/>
@@ -3057,16 +3053,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B79" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C79" s="35" t="str">
-        <x:v>posterior_cingulate_gyrus</x:v>
+        <x:v>postcentral_gyrus</x:v>
       </x:c>
       <x:c r="D79" s="35" t="str">
-        <x:v>Posterior cingulate gyrus</x:v>
+        <x:v>Postcentral gyrus</x:v>
       </x:c>
       <x:c r="E79" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F79" s="35" t="str">
         <x:v>yes</x:v>
@@ -3078,7 +3074,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I79" s="35" t="str">
-        <x:v>annotations/021_posterior_cingulate_gyrus.nii.gz</x:v>
+        <x:v>annotations/020_postcentral_gyrus.nii.gz</x:v>
       </x:c>
       <x:c r="J79" s="35" t="str"/>
       <x:c r="K79" s="35" t="str"/>
@@ -3092,20 +3088,26 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C80" s="35" t="str">
-        <x:v>posterior_commissure</x:v>
+        <x:v>posterior_cingulate_gyrus</x:v>
       </x:c>
       <x:c r="D80" s="35" t="str">
-        <x:v>Posterior commissure</x:v>
+        <x:v>Posterior cingulate gyrus</x:v>
       </x:c>
       <x:c r="E80" s="35" t="str">
-        <x:v>white_matter; midline; brainstem</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="F80" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G80" s="35" t="str"/>
-      <x:c r="H80" s="35" t="str"/>
-      <x:c r="I80" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G80" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H80" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I80" s="35" t="str">
+        <x:v>annotations/021_posterior_cingulate_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J80" s="35" t="str"/>
       <x:c r="K80" s="35" t="str"/>
       <x:c r="L80" s="36" t="str"/>
@@ -3115,16 +3117,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B81" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C81" s="35" t="str">
-        <x:v>posterior_limb_of_the_internal_capsule</x:v>
+        <x:v>posterior_commissure</x:v>
       </x:c>
       <x:c r="D81" s="35" t="str">
-        <x:v>Posterior limb of the internal capsule</x:v>
+        <x:v>Posterior commissure</x:v>
       </x:c>
       <x:c r="E81" s="35" t="str">
-        <x:v>white_matter; basal_ganglia</x:v>
+        <x:v>white_matter; midline; brainstem</x:v>
       </x:c>
       <x:c r="F81" s="35" t="str">
         <x:v>no</x:v>
@@ -3144,26 +3146,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C82" s="35" t="str">
-        <x:v>precentral_gyrus</x:v>
+        <x:v>posterior_limb_of_the_internal_capsule</x:v>
       </x:c>
       <x:c r="D82" s="35" t="str">
-        <x:v>Precentral gyrus</x:v>
+        <x:v>Posterior limb of the internal capsule</x:v>
       </x:c>
       <x:c r="E82" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>white_matter; basal_ganglia</x:v>
       </x:c>
       <x:c r="F82" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G82" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H82" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I82" s="35" t="str">
-        <x:v>annotations/022_precentral_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G82" s="35" t="str"/>
+      <x:c r="H82" s="35" t="str"/>
+      <x:c r="I82" s="35" t="str"/>
       <x:c r="J82" s="35" t="str"/>
       <x:c r="K82" s="35" t="str"/>
       <x:c r="L82" s="36" t="str"/>
@@ -3173,13 +3169,13 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B83" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C83" s="35" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>precentral_gyrus</x:v>
       </x:c>
       <x:c r="D83" s="35" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>Precentral gyrus</x:v>
       </x:c>
       <x:c r="E83" s="35" t="str">
         <x:v>cortex</x:v>
@@ -3194,7 +3190,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I83" s="35" t="str">
-        <x:v>annotations/023_precuneus.nii.gz</x:v>
+        <x:v>annotations/022_precentral_gyrus.nii.gz</x:v>
       </x:c>
       <x:c r="J83" s="35" t="str"/>
       <x:c r="K83" s="35" t="str"/>
@@ -3205,23 +3201,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B84" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C84" s="35" t="str">
-        <x:v>premedullary_cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="D84" s="35" t="str">
-        <x:v>Premedullary cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="E84" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F84" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G84" s="35" t="str"/>
-      <x:c r="H84" s="35" t="str"/>
-      <x:c r="I84" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G84" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H84" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I84" s="35" t="str">
+        <x:v>annotations/023_precuneus.nii.gz</x:v>
+      </x:c>
       <x:c r="J84" s="35" t="str"/>
       <x:c r="K84" s="35" t="str"/>
       <x:c r="L84" s="36" t="str"/>
@@ -3234,10 +3236,10 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C85" s="35" t="str">
-        <x:v>prepontine_cistern</x:v>
+        <x:v>premedullary_cistern</x:v>
       </x:c>
       <x:c r="D85" s="35" t="str">
-        <x:v>Prepontine cistern</x:v>
+        <x:v>Premedullary cistern</x:v>
       </x:c>
       <x:c r="E85" s="35" t="str">
         <x:v>csf_spaces; brainstem</x:v>
@@ -3260,26 +3262,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C86" s="35" t="str">
-        <x:v>putamen</x:v>
+        <x:v>prepontine_cistern</x:v>
       </x:c>
       <x:c r="D86" s="35" t="str">
-        <x:v>Putamen</x:v>
+        <x:v>Prepontine cistern</x:v>
       </x:c>
       <x:c r="E86" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F86" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G86" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H86" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I86" s="35" t="str">
-        <x:v>annotations/004_putamen.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G86" s="35" t="str"/>
+      <x:c r="H86" s="35" t="str"/>
+      <x:c r="I86" s="35" t="str"/>
       <x:c r="J86" s="35" t="str"/>
       <x:c r="K86" s="35" t="str"/>
       <x:c r="L86" s="36" t="str"/>
@@ -3292,20 +3288,26 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C87" s="35" t="str">
-        <x:v>quadrigeminal_cistern</x:v>
+        <x:v>putamen</x:v>
       </x:c>
       <x:c r="D87" s="35" t="str">
-        <x:v>Quadrigeminal cistern</x:v>
+        <x:v>Putamen</x:v>
       </x:c>
       <x:c r="E87" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="F87" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G87" s="35" t="str"/>
-      <x:c r="H87" s="35" t="str"/>
-      <x:c r="I87" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G87" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H87" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I87" s="35" t="str">
+        <x:v>annotations/004_putamen.nii.gz</x:v>
+      </x:c>
       <x:c r="J87" s="35" t="str"/>
       <x:c r="K87" s="35" t="str"/>
       <x:c r="L87" s="36" t="str"/>
@@ -3318,26 +3320,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C88" s="35" t="str">
-        <x:v>septum_pellucidum</x:v>
+        <x:v>quadrigeminal_cistern</x:v>
       </x:c>
       <x:c r="D88" s="35" t="str">
-        <x:v>Septum pellucidum</x:v>
+        <x:v>Quadrigeminal cistern</x:v>
       </x:c>
       <x:c r="E88" s="35" t="str">
-        <x:v>midline; ventricles; csf_spaces</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F88" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G88" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H88" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I88" s="35" t="str">
-        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G88" s="35" t="str"/>
+      <x:c r="H88" s="35" t="str"/>
+      <x:c r="I88" s="35" t="str"/>
       <x:c r="J88" s="35" t="str"/>
       <x:c r="K88" s="35" t="str"/>
       <x:c r="L88" s="36" t="str"/>
@@ -3350,13 +3346,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
-        <x:v>splenium_of_the_corpus_callosum</x:v>
+        <x:v>septum_pellucidum</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>Splenium of the corpus callosum</x:v>
+        <x:v>Septum pellucidum</x:v>
       </x:c>
       <x:c r="E89" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F89" s="35" t="str">
         <x:v>yes</x:v>
@@ -3368,7 +3364,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I89" s="35" t="str">
-        <x:v>annotations/075_splenium_of_the_corpus_callosum.nii.gz</x:v>
+        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
       </x:c>
       <x:c r="J89" s="35" t="str"/>
       <x:c r="K89" s="35" t="str"/>
@@ -3382,57 +3378,57 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
-        <x:v>subthalamic_region</x:v>
+        <x:v>splenium_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>Subthalamic region</x:v>
+        <x:v>Splenium of the corpus callosum</x:v>
       </x:c>
       <x:c r="E90" s="35" t="str">
-        <x:v>deep_gray; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F90" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G90" s="35" t="str"/>
-      <x:c r="H90" s="35" t="str"/>
-      <x:c r="I90" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G90" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H90" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I90" s="35" t="str">
+        <x:v>annotations/075_splenium_of_the_corpus_callosum.nii.gz</x:v>
+      </x:c>
       <x:c r="J90" s="35" t="str"/>
       <x:c r="K90" s="35" t="str"/>
-      <x:c r="L90" s="36" t="str">
-        <x:v>Optional beginner-to-intermediate deep gray landmark if it can be shown cleanly on this T1.</x:v>
-      </x:c>
+      <x:c r="L90" s="36" t="str"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B91" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
-        <x:v>superior_frontal_gyrus</x:v>
+        <x:v>subthalamic_region</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>Superior frontal gyrus</x:v>
+        <x:v>Subthalamic region</x:v>
       </x:c>
       <x:c r="E91" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>deep_gray; basal_ganglia</x:v>
       </x:c>
       <x:c r="F91" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G91" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H91" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I91" s="35" t="str">
-        <x:v>annotations/024_superior_frontal_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G91" s="35" t="str"/>
+      <x:c r="H91" s="35" t="str"/>
+      <x:c r="I91" s="35" t="str"/>
       <x:c r="J91" s="35" t="str"/>
       <x:c r="K91" s="35" t="str"/>
-      <x:c r="L91" s="36" t="str"/>
+      <x:c r="L91" s="36" t="str">
+        <x:v>Optional beginner-to-intermediate deep gray landmark if it can be shown cleanly on this T1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="33" t="str">
@@ -3442,39 +3438,45 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
-        <x:v>superior_orbital_fissure</x:v>
+        <x:v>superior_frontal_gyrus</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>Superior orbital fissure</x:v>
+        <x:v>Superior frontal gyrus</x:v>
       </x:c>
       <x:c r="E92" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F92" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G92" s="35" t="str"/>
-      <x:c r="H92" s="35" t="str"/>
-      <x:c r="I92" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G92" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H92" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I92" s="35" t="str">
+        <x:v>annotations/024_superior_frontal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J92" s="35" t="str"/>
       <x:c r="K92" s="35" t="str"/>
       <x:c r="L92" s="36" t="str"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B93" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
-        <x:v>superior_temporal_gyrus</x:v>
+        <x:v>superior_orbital_fissure</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>Superior temporal gyrus</x:v>
+        <x:v>Superior orbital fissure</x:v>
       </x:c>
       <x:c r="E93" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="F93" s="35" t="str">
         <x:v>no</x:v>
@@ -3488,32 +3490,26 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B94" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
-        <x:v>supramarginal_gyrus</x:v>
+        <x:v>superior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="D94" s="35" t="str">
-        <x:v>Supramarginal gyrus</x:v>
+        <x:v>Superior temporal gyrus</x:v>
       </x:c>
       <x:c r="E94" s="35" t="str">
         <x:v>cortex</x:v>
       </x:c>
       <x:c r="F94" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G94" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H94" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I94" s="35" t="str">
-        <x:v>annotations/025_supramarginal_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G94" s="35" t="str"/>
+      <x:c r="H94" s="35" t="str"/>
+      <x:c r="I94" s="35" t="str"/>
       <x:c r="J94" s="35" t="str"/>
       <x:c r="K94" s="35" t="str"/>
       <x:c r="L94" s="36" t="str"/>
@@ -3523,23 +3519,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B95" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C95" s="35" t="str">
-        <x:v>suprasellar_cistern</x:v>
+        <x:v>supramarginal_gyrus</x:v>
       </x:c>
       <x:c r="D95" s="35" t="str">
-        <x:v>Suprasellar cistern</x:v>
+        <x:v>Supramarginal gyrus</x:v>
       </x:c>
       <x:c r="E95" s="35" t="str">
-        <x:v>csf_spaces; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F95" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G95" s="35" t="str"/>
-      <x:c r="H95" s="35" t="str"/>
-      <x:c r="I95" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G95" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H95" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I95" s="35" t="str">
+        <x:v>annotations/025_supramarginal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J95" s="35" t="str"/>
       <x:c r="K95" s="35" t="str"/>
       <x:c r="L95" s="36" t="str"/>
@@ -3552,26 +3554,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C96" s="35" t="str">
-        <x:v>sylvian_fissure</x:v>
+        <x:v>suprasellar_cistern</x:v>
       </x:c>
       <x:c r="D96" s="35" t="str">
-        <x:v>Sylvian fissure</x:v>
+        <x:v>Suprasellar cistern</x:v>
       </x:c>
       <x:c r="E96" s="35" t="str">
-        <x:v>csf_spaces; cortex</x:v>
+        <x:v>csf_spaces; skull_base</x:v>
       </x:c>
       <x:c r="F96" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G96" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H96" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I96" s="35" t="str">
-        <x:v>annotations/051_sylvian_fissure.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G96" s="35" t="str"/>
+      <x:c r="H96" s="35" t="str"/>
+      <x:c r="I96" s="35" t="str"/>
       <x:c r="J96" s="35" t="str"/>
       <x:c r="K96" s="35" t="str"/>
       <x:c r="L96" s="36" t="str"/>
@@ -3584,13 +3580,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C97" s="35" t="str">
-        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>sylvian_fissure</x:v>
       </x:c>
       <x:c r="D97" s="35" t="str">
-        <x:v>Temporal horn of the lateral ventricle</x:v>
+        <x:v>Sylvian fissure</x:v>
       </x:c>
       <x:c r="E97" s="35" t="str">
-        <x:v>ventricles; csf_spaces; deep_gray</x:v>
+        <x:v>csf_spaces; cortex</x:v>
       </x:c>
       <x:c r="F97" s="35" t="str">
         <x:v>yes</x:v>
@@ -3602,7 +3598,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I97" s="35" t="str">
-        <x:v>annotations/045_temporal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/051_sylvian_fissure.nii.gz</x:v>
       </x:c>
       <x:c r="J97" s="35" t="str"/>
       <x:c r="K97" s="35" t="str"/>
@@ -3616,80 +3612,86 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C98" s="35" t="str">
-        <x:v>temporal_lobe</x:v>
+        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D98" s="35" t="str">
-        <x:v>Temporal lobe</x:v>
+        <x:v>Temporal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E98" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces; deep_gray</x:v>
       </x:c>
       <x:c r="F98" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G98" s="35" t="str"/>
-      <x:c r="H98" s="35" t="str"/>
-      <x:c r="I98" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G98" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H98" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I98" s="35" t="str">
+        <x:v>annotations/045_temporal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J98" s="35" t="str"/>
       <x:c r="K98" s="35" t="str"/>
-      <x:c r="L98" s="36" t="str">
-        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
-      </x:c>
+      <x:c r="L98" s="36" t="str"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B99" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C99" s="35" t="str">
-        <x:v>temporal_pole</x:v>
+        <x:v>temporal_lobe</x:v>
       </x:c>
       <x:c r="D99" s="35" t="str">
-        <x:v>Temporal pole</x:v>
+        <x:v>Temporal lobe</x:v>
       </x:c>
       <x:c r="E99" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="F99" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G99" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H99" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I99" s="35" t="str">
-        <x:v>annotations/026_temporal_pole.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G99" s="35" t="str"/>
+      <x:c r="H99" s="35" t="str"/>
+      <x:c r="I99" s="35" t="str"/>
       <x:c r="J99" s="35" t="str"/>
       <x:c r="K99" s="35" t="str"/>
-      <x:c r="L99" s="36" t="str"/>
+      <x:c r="L99" s="36" t="str">
+        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
+      </x:c>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B100" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C100" s="35" t="str">
-        <x:v>tentorium_cerebelli</x:v>
+        <x:v>temporal_pole</x:v>
       </x:c>
       <x:c r="D100" s="35" t="str">
-        <x:v>Tentorium cerebelli</x:v>
+        <x:v>Temporal pole</x:v>
       </x:c>
       <x:c r="E100" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F100" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G100" s="35" t="str"/>
-      <x:c r="H100" s="35" t="str"/>
-      <x:c r="I100" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G100" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H100" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I100" s="35" t="str">
+        <x:v>annotations/026_temporal_pole.nii.gz</x:v>
+      </x:c>
       <x:c r="J100" s="35" t="str"/>
       <x:c r="K100" s="35" t="str"/>
       <x:c r="L100" s="36" t="str"/>
@@ -3702,26 +3704,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C101" s="35" t="str">
-        <x:v>thalamus</x:v>
+        <x:v>tentorium_cerebelli</x:v>
       </x:c>
       <x:c r="D101" s="35" t="str">
-        <x:v>Thalamus</x:v>
+        <x:v>Tentorium cerebelli</x:v>
       </x:c>
       <x:c r="E101" s="35" t="str">
-        <x:v>deep_gray</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="F101" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G101" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H101" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I101" s="35" t="str">
-        <x:v>annotations/002_thalamus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G101" s="35" t="str"/>
+      <x:c r="H101" s="35" t="str"/>
+      <x:c r="I101" s="35" t="str"/>
       <x:c r="J101" s="35" t="str"/>
       <x:c r="K101" s="35" t="str"/>
       <x:c r="L101" s="36" t="str"/>
@@ -3734,13 +3730,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C102" s="35" t="str">
-        <x:v>third_ventricle</x:v>
+        <x:v>thalamus</x:v>
       </x:c>
       <x:c r="D102" s="35" t="str">
-        <x:v>Third ventricle</x:v>
+        <x:v>Thalamus</x:v>
       </x:c>
       <x:c r="E102" s="35" t="str">
-        <x:v>ventricles; csf_spaces; midline</x:v>
+        <x:v>deep_gray</x:v>
       </x:c>
       <x:c r="F102" s="35" t="str">
         <x:v>yes</x:v>
@@ -3752,7 +3748,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I102" s="35" t="str">
-        <x:v>annotations/006_third_ventricle.nii.gz</x:v>
+        <x:v>annotations/002_thalamus.nii.gz</x:v>
       </x:c>
       <x:c r="J102" s="35" t="str"/>
       <x:c r="K102" s="35" t="str"/>
@@ -3766,25 +3762,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C103" s="35" t="str">
-        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
+        <x:v>third_ventricle</x:v>
       </x:c>
       <x:c r="D103" s="35" t="str">
-        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
+        <x:v>Third ventricle</x:v>
       </x:c>
       <x:c r="E103" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; midline</x:v>
       </x:c>
       <x:c r="F103" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G103" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H103" s="35" t="str">
-        <x:v>accepted</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I103" s="35" t="str">
-        <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/006_third_ventricle.nii.gz</x:v>
       </x:c>
       <x:c r="J103" s="35" t="str"/>
       <x:c r="K103" s="35" t="str"/>
@@ -3795,65 +3791,97 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B104" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C104" s="35" t="str">
-        <x:v>uncus</x:v>
+        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D104" s="35" t="str">
-        <x:v>Uncus</x:v>
+        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E104" s="35" t="str">
-        <x:v>limbic; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F104" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G104" s="35" t="str"/>
-      <x:c r="H104" s="35" t="str"/>
-      <x:c r="I104" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G104" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H104" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I104" s="35" t="str">
+        <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J104" s="35" t="str"/>
       <x:c r="K104" s="35" t="str"/>
       <x:c r="L104" s="36" t="str"/>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="37" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="B105" s="38" t="str">
-        <x:v>advanced</x:v>
-      </x:c>
-      <x:c r="C105" s="39" t="str">
+      <x:c r="A105" s="33" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="B105" s="34" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="C105" s="35" t="str">
+        <x:v>uncus</x:v>
+      </x:c>
+      <x:c r="D105" s="35" t="str">
+        <x:v>Uncus</x:v>
+      </x:c>
+      <x:c r="E105" s="35" t="str">
+        <x:v>limbic; cortex</x:v>
+      </x:c>
+      <x:c r="F105" s="35" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G105" s="35" t="str"/>
+      <x:c r="H105" s="35" t="str"/>
+      <x:c r="I105" s="35" t="str"/>
+      <x:c r="J105" s="35" t="str"/>
+      <x:c r="K105" s="35" t="str"/>
+      <x:c r="L105" s="36" t="str"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="37" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="B106" s="38" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="C106" s="39" t="str">
         <x:v>vermis</x:v>
       </x:c>
-      <x:c r="D105" s="39" t="str">
+      <x:c r="D106" s="39" t="str">
         <x:v>Vermis</x:v>
       </x:c>
-      <x:c r="E105" s="39" t="str">
+      <x:c r="E106" s="39" t="str">
         <x:v>cerebellum; midline</x:v>
       </x:c>
-      <x:c r="F105" s="39" t="str">
+      <x:c r="F106" s="39" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="G105" s="39" t="str"/>
-      <x:c r="H105" s="39" t="str"/>
-      <x:c r="I105" s="39" t="str"/>
-      <x:c r="J105" s="39" t="str"/>
-      <x:c r="K105" s="39" t="str"/>
-      <x:c r="L105" s="40" t="str"/>
+      <x:c r="G106" s="39" t="str"/>
+      <x:c r="H106" s="39" t="str"/>
+      <x:c r="I106" s="39" t="str"/>
+      <x:c r="J106" s="39" t="str"/>
+      <x:c r="K106" s="39" t="str"/>
+      <x:c r="L106" s="40" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="A2:A105">
+    <x:dataValidation type="list" sqref="A2:A106">
       <x:formula1>"yes,no"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="B2:B105">
+    <x:dataValidation type="list" sqref="B2:B106">
       <x:formula1>"beginner,advanced"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8de694d75a0e4ad3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6edf86a302a14020"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5438,16 +5466,16 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="45" t="str">
-        <x:v>orbitofrontal_cortex</x:v>
+        <x:v>optic_nerve</x:v>
       </x:c>
       <x:c r="B68" s="35" t="str">
-        <x:v>Orbitofrontal cortex</x:v>
+        <x:v>Optic nerve</x:v>
       </x:c>
       <x:c r="C68" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D68" s="35" t="str">
-        <x:v>cortex; skull_base</x:v>
+        <x:v>cranial_nerves; skull_base; orbit</x:v>
       </x:c>
       <x:c r="E68" s="34" t="str"/>
       <x:c r="F68" s="34" t="str"/>
@@ -5461,16 +5489,16 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="45" t="str">
-        <x:v>parahippocampal_gyrus</x:v>
+        <x:v>orbitofrontal_cortex</x:v>
       </x:c>
       <x:c r="B69" s="35" t="str">
-        <x:v>Parahippocampal gyrus</x:v>
+        <x:v>Orbitofrontal cortex</x:v>
       </x:c>
       <x:c r="C69" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D69" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex; skull_base</x:v>
       </x:c>
       <x:c r="E69" s="34" t="str"/>
       <x:c r="F69" s="34" t="str"/>
@@ -5484,16 +5512,16 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="45" t="str">
-        <x:v>parietal_lobe</x:v>
+        <x:v>parahippocampal_gyrus</x:v>
       </x:c>
       <x:c r="B70" s="35" t="str">
-        <x:v>Parietal lobe</x:v>
+        <x:v>Parahippocampal gyrus</x:v>
       </x:c>
       <x:c r="C70" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D70" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="E70" s="34" t="str"/>
       <x:c r="F70" s="34" t="str"/>
@@ -5507,16 +5535,16 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="45" t="str">
-        <x:v>parieto_occipital_sulcus</x:v>
+        <x:v>parietal_lobe</x:v>
       </x:c>
       <x:c r="B71" s="35" t="str">
-        <x:v>Parieto-occipital sulcus</x:v>
+        <x:v>Parietal lobe</x:v>
       </x:c>
       <x:c r="C71" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D71" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="E71" s="34" t="str"/>
       <x:c r="F71" s="34" t="str"/>
@@ -5530,10 +5558,10 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="45" t="str">
-        <x:v>pars_opercularis</x:v>
+        <x:v>parieto_occipital_sulcus</x:v>
       </x:c>
       <x:c r="B72" s="35" t="str">
-        <x:v>Pars opercularis</x:v>
+        <x:v>Parieto-occipital sulcus</x:v>
       </x:c>
       <x:c r="C72" s="35" t="str">
         <x:v>advanced</x:v>
@@ -5553,10 +5581,10 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="45" t="str">
-        <x:v>pars_orbitalis</x:v>
+        <x:v>pars_opercularis</x:v>
       </x:c>
       <x:c r="B73" s="35" t="str">
-        <x:v>Pars orbitalis</x:v>
+        <x:v>Pars opercularis</x:v>
       </x:c>
       <x:c r="C73" s="35" t="str">
         <x:v>advanced</x:v>
@@ -5576,10 +5604,10 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="45" t="str">
-        <x:v>pars_triangularis</x:v>
+        <x:v>pars_orbitalis</x:v>
       </x:c>
       <x:c r="B74" s="35" t="str">
-        <x:v>Pars triangularis</x:v>
+        <x:v>Pars orbitalis</x:v>
       </x:c>
       <x:c r="C74" s="35" t="str">
         <x:v>advanced</x:v>
@@ -5599,16 +5627,16 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="45" t="str">
-        <x:v>pineal_gland</x:v>
+        <x:v>pars_triangularis</x:v>
       </x:c>
       <x:c r="B75" s="35" t="str">
-        <x:v>Pineal gland</x:v>
+        <x:v>Pars triangularis</x:v>
       </x:c>
       <x:c r="C75" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D75" s="35" t="str">
-        <x:v>midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E75" s="34" t="str"/>
       <x:c r="F75" s="34" t="str"/>
@@ -5622,16 +5650,16 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="45" t="str">
-        <x:v>pituitary_fossa</x:v>
+        <x:v>pineal_gland</x:v>
       </x:c>
       <x:c r="B76" s="35" t="str">
-        <x:v>Pituitary fossa</x:v>
+        <x:v>Pineal gland</x:v>
       </x:c>
       <x:c r="C76" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D76" s="35" t="str">
-        <x:v>skull_base; midline</x:v>
+        <x:v>midline</x:v>
       </x:c>
       <x:c r="E76" s="34" t="str"/>
       <x:c r="F76" s="34" t="str"/>
@@ -5645,16 +5673,16 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="45" t="str">
-        <x:v>pons</x:v>
+        <x:v>pituitary_fossa</x:v>
       </x:c>
       <x:c r="B77" s="35" t="str">
-        <x:v>Pons</x:v>
+        <x:v>Pituitary fossa</x:v>
       </x:c>
       <x:c r="C77" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D77" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>skull_base; midline</x:v>
       </x:c>
       <x:c r="E77" s="34" t="str"/>
       <x:c r="F77" s="34" t="str"/>
@@ -5668,16 +5696,16 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="45" t="str">
-        <x:v>postcentral_gyrus</x:v>
+        <x:v>pons</x:v>
       </x:c>
       <x:c r="B78" s="35" t="str">
-        <x:v>Postcentral gyrus</x:v>
+        <x:v>Pons</x:v>
       </x:c>
       <x:c r="C78" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D78" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="E78" s="34" t="str"/>
       <x:c r="F78" s="34" t="str"/>
@@ -5691,16 +5719,16 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="45" t="str">
-        <x:v>posterior_cingulate_gyrus</x:v>
+        <x:v>postcentral_gyrus</x:v>
       </x:c>
       <x:c r="B79" s="35" t="str">
-        <x:v>Posterior cingulate gyrus</x:v>
+        <x:v>Postcentral gyrus</x:v>
       </x:c>
       <x:c r="C79" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D79" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E79" s="34" t="str"/>
       <x:c r="F79" s="34" t="str"/>
@@ -5714,16 +5742,16 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="45" t="str">
-        <x:v>posterior_commissure</x:v>
+        <x:v>posterior_cingulate_gyrus</x:v>
       </x:c>
       <x:c r="B80" s="35" t="str">
-        <x:v>Posterior commissure</x:v>
+        <x:v>Posterior cingulate gyrus</x:v>
       </x:c>
       <x:c r="C80" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D80" s="35" t="str">
-        <x:v>white_matter; midline; brainstem</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="E80" s="34" t="str"/>
       <x:c r="F80" s="34" t="str"/>
@@ -5737,16 +5765,16 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="45" t="str">
-        <x:v>posterior_limb_of_the_internal_capsule</x:v>
+        <x:v>posterior_commissure</x:v>
       </x:c>
       <x:c r="B81" s="35" t="str">
-        <x:v>Posterior limb of the internal capsule</x:v>
+        <x:v>Posterior commissure</x:v>
       </x:c>
       <x:c r="C81" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D81" s="35" t="str">
-        <x:v>white_matter; basal_ganglia</x:v>
+        <x:v>white_matter; midline; brainstem</x:v>
       </x:c>
       <x:c r="E81" s="34" t="str"/>
       <x:c r="F81" s="34" t="str"/>
@@ -5760,16 +5788,16 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="45" t="str">
-        <x:v>precentral_gyrus</x:v>
+        <x:v>posterior_limb_of_the_internal_capsule</x:v>
       </x:c>
       <x:c r="B82" s="35" t="str">
-        <x:v>Precentral gyrus</x:v>
+        <x:v>Posterior limb of the internal capsule</x:v>
       </x:c>
       <x:c r="C82" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D82" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>white_matter; basal_ganglia</x:v>
       </x:c>
       <x:c r="E82" s="34" t="str"/>
       <x:c r="F82" s="34" t="str"/>
@@ -5783,13 +5811,13 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="45" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>precentral_gyrus</x:v>
       </x:c>
       <x:c r="B83" s="35" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>Precentral gyrus</x:v>
       </x:c>
       <x:c r="C83" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D83" s="35" t="str">
         <x:v>cortex</x:v>
@@ -5806,16 +5834,16 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="45" t="str">
-        <x:v>premedullary_cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="B84" s="35" t="str">
-        <x:v>Premedullary cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="C84" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D84" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E84" s="34" t="str"/>
       <x:c r="F84" s="34" t="str"/>
@@ -5829,10 +5857,10 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="45" t="str">
-        <x:v>prepontine_cistern</x:v>
+        <x:v>premedullary_cistern</x:v>
       </x:c>
       <x:c r="B85" s="35" t="str">
-        <x:v>Prepontine cistern</x:v>
+        <x:v>Premedullary cistern</x:v>
       </x:c>
       <x:c r="C85" s="35" t="str">
         <x:v>beginner</x:v>
@@ -5852,16 +5880,16 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="45" t="str">
-        <x:v>putamen</x:v>
+        <x:v>prepontine_cistern</x:v>
       </x:c>
       <x:c r="B86" s="35" t="str">
-        <x:v>Putamen</x:v>
+        <x:v>Prepontine cistern</x:v>
       </x:c>
       <x:c r="C86" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D86" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E86" s="34" t="str"/>
       <x:c r="F86" s="34" t="str"/>
@@ -5875,16 +5903,16 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="45" t="str">
-        <x:v>quadrigeminal_cistern</x:v>
+        <x:v>putamen</x:v>
       </x:c>
       <x:c r="B87" s="35" t="str">
-        <x:v>Quadrigeminal cistern</x:v>
+        <x:v>Putamen</x:v>
       </x:c>
       <x:c r="C87" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D87" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="E87" s="34" t="str"/>
       <x:c r="F87" s="34" t="str"/>
@@ -5898,16 +5926,16 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="45" t="str">
-        <x:v>septum_pellucidum</x:v>
+        <x:v>quadrigeminal_cistern</x:v>
       </x:c>
       <x:c r="B88" s="35" t="str">
-        <x:v>Septum pellucidum</x:v>
+        <x:v>Quadrigeminal cistern</x:v>
       </x:c>
       <x:c r="C88" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D88" s="35" t="str">
-        <x:v>midline; ventricles; csf_spaces</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E88" s="34" t="str"/>
       <x:c r="F88" s="34" t="str"/>
@@ -5921,16 +5949,16 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="45" t="str">
-        <x:v>splenium_of_the_corpus_callosum</x:v>
+        <x:v>septum_pellucidum</x:v>
       </x:c>
       <x:c r="B89" s="35" t="str">
-        <x:v>Splenium of the corpus callosum</x:v>
+        <x:v>Septum pellucidum</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E89" s="34" t="str"/>
       <x:c r="F89" s="34" t="str"/>
@@ -5944,16 +5972,16 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="45" t="str">
-        <x:v>subthalamic_region</x:v>
+        <x:v>splenium_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="B90" s="35" t="str">
-        <x:v>Subthalamic region</x:v>
+        <x:v>Splenium of the corpus callosum</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>deep_gray; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E90" s="34" t="str"/>
       <x:c r="F90" s="34" t="str"/>
@@ -5967,16 +5995,16 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="45" t="str">
-        <x:v>superior_frontal_gyrus</x:v>
+        <x:v>subthalamic_region</x:v>
       </x:c>
       <x:c r="B91" s="35" t="str">
-        <x:v>Superior frontal gyrus</x:v>
+        <x:v>Subthalamic region</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>deep_gray; basal_ganglia</x:v>
       </x:c>
       <x:c r="E91" s="34" t="str"/>
       <x:c r="F91" s="34" t="str"/>
@@ -5990,16 +6018,16 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="45" t="str">
-        <x:v>superior_orbital_fissure</x:v>
+        <x:v>superior_frontal_gyrus</x:v>
       </x:c>
       <x:c r="B92" s="35" t="str">
-        <x:v>Superior orbital fissure</x:v>
+        <x:v>Superior frontal gyrus</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E92" s="34" t="str"/>
       <x:c r="F92" s="34" t="str"/>
@@ -6013,16 +6041,16 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="45" t="str">
-        <x:v>superior_temporal_gyrus</x:v>
+        <x:v>superior_orbital_fissure</x:v>
       </x:c>
       <x:c r="B93" s="35" t="str">
-        <x:v>Superior temporal gyrus</x:v>
+        <x:v>Superior orbital fissure</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="E93" s="34" t="str"/>
       <x:c r="F93" s="34" t="str"/>
@@ -6036,13 +6064,13 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="45" t="str">
-        <x:v>supramarginal_gyrus</x:v>
+        <x:v>superior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="B94" s="35" t="str">
-        <x:v>Supramarginal gyrus</x:v>
+        <x:v>Superior temporal gyrus</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D94" s="35" t="str">
         <x:v>cortex</x:v>
@@ -6059,16 +6087,16 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="45" t="str">
-        <x:v>suprasellar_cistern</x:v>
+        <x:v>supramarginal_gyrus</x:v>
       </x:c>
       <x:c r="B95" s="35" t="str">
-        <x:v>Suprasellar cistern</x:v>
+        <x:v>Supramarginal gyrus</x:v>
       </x:c>
       <x:c r="C95" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D95" s="35" t="str">
-        <x:v>csf_spaces; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E95" s="34" t="str"/>
       <x:c r="F95" s="34" t="str"/>
@@ -6082,16 +6110,16 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="45" t="str">
-        <x:v>sylvian_fissure</x:v>
+        <x:v>suprasellar_cistern</x:v>
       </x:c>
       <x:c r="B96" s="35" t="str">
-        <x:v>Sylvian fissure</x:v>
+        <x:v>Suprasellar cistern</x:v>
       </x:c>
       <x:c r="C96" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D96" s="35" t="str">
-        <x:v>csf_spaces; cortex</x:v>
+        <x:v>csf_spaces; skull_base</x:v>
       </x:c>
       <x:c r="E96" s="34" t="str"/>
       <x:c r="F96" s="34" t="str"/>
@@ -6105,16 +6133,16 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="45" t="str">
-        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>sylvian_fissure</x:v>
       </x:c>
       <x:c r="B97" s="35" t="str">
-        <x:v>Temporal horn of the lateral ventricle</x:v>
+        <x:v>Sylvian fissure</x:v>
       </x:c>
       <x:c r="C97" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D97" s="35" t="str">
-        <x:v>ventricles; csf_spaces; deep_gray</x:v>
+        <x:v>csf_spaces; cortex</x:v>
       </x:c>
       <x:c r="E97" s="34" t="str"/>
       <x:c r="F97" s="34" t="str"/>
@@ -6128,16 +6156,16 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="45" t="str">
-        <x:v>temporal_lobe</x:v>
+        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B98" s="35" t="str">
-        <x:v>Temporal lobe</x:v>
+        <x:v>Temporal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C98" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D98" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces; deep_gray</x:v>
       </x:c>
       <x:c r="E98" s="34" t="str"/>
       <x:c r="F98" s="34" t="str"/>
@@ -6151,16 +6179,16 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="45" t="str">
-        <x:v>temporal_pole</x:v>
+        <x:v>temporal_lobe</x:v>
       </x:c>
       <x:c r="B99" s="35" t="str">
-        <x:v>Temporal pole</x:v>
+        <x:v>Temporal lobe</x:v>
       </x:c>
       <x:c r="C99" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D99" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="E99" s="34" t="str"/>
       <x:c r="F99" s="34" t="str"/>
@@ -6174,16 +6202,16 @@
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="45" t="str">
-        <x:v>tentorium_cerebelli</x:v>
+        <x:v>temporal_pole</x:v>
       </x:c>
       <x:c r="B100" s="35" t="str">
-        <x:v>Tentorium cerebelli</x:v>
+        <x:v>Temporal pole</x:v>
       </x:c>
       <x:c r="C100" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D100" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E100" s="34" t="str"/>
       <x:c r="F100" s="34" t="str"/>
@@ -6197,16 +6225,16 @@
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="45" t="str">
-        <x:v>thalamus</x:v>
+        <x:v>tentorium_cerebelli</x:v>
       </x:c>
       <x:c r="B101" s="35" t="str">
-        <x:v>Thalamus</x:v>
+        <x:v>Tentorium cerebelli</x:v>
       </x:c>
       <x:c r="C101" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D101" s="35" t="str">
-        <x:v>deep_gray</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="E101" s="34" t="str"/>
       <x:c r="F101" s="34" t="str"/>
@@ -6220,16 +6248,16 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="45" t="str">
-        <x:v>third_ventricle</x:v>
+        <x:v>thalamus</x:v>
       </x:c>
       <x:c r="B102" s="35" t="str">
-        <x:v>Third ventricle</x:v>
+        <x:v>Thalamus</x:v>
       </x:c>
       <x:c r="C102" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D102" s="35" t="str">
-        <x:v>ventricles; csf_spaces; midline</x:v>
+        <x:v>deep_gray</x:v>
       </x:c>
       <x:c r="E102" s="34" t="str"/>
       <x:c r="F102" s="34" t="str"/>
@@ -6243,16 +6271,16 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="45" t="str">
-        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
+        <x:v>third_ventricle</x:v>
       </x:c>
       <x:c r="B103" s="35" t="str">
-        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
+        <x:v>Third ventricle</x:v>
       </x:c>
       <x:c r="C103" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D103" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; midline</x:v>
       </x:c>
       <x:c r="E103" s="34" t="str"/>
       <x:c r="F103" s="34" t="str"/>
@@ -6266,16 +6294,16 @@
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="45" t="str">
-        <x:v>uncus</x:v>
+        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B104" s="35" t="str">
-        <x:v>Uncus</x:v>
+        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C104" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D104" s="35" t="str">
-        <x:v>limbic; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E104" s="34" t="str"/>
       <x:c r="F104" s="34" t="str"/>
@@ -6288,32 +6316,55 @@
       <x:c r="M104" s="36" t="str"/>
     </x:row>
     <x:row r="105">
-      <x:c r="A105" s="46" t="str">
+      <x:c r="A105" s="45" t="str">
+        <x:v>uncus</x:v>
+      </x:c>
+      <x:c r="B105" s="35" t="str">
+        <x:v>Uncus</x:v>
+      </x:c>
+      <x:c r="C105" s="35" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="D105" s="35" t="str">
+        <x:v>limbic; cortex</x:v>
+      </x:c>
+      <x:c r="E105" s="34" t="str"/>
+      <x:c r="F105" s="34" t="str"/>
+      <x:c r="G105" s="34" t="str"/>
+      <x:c r="H105" s="34" t="str"/>
+      <x:c r="I105" s="34" t="str"/>
+      <x:c r="J105" s="34" t="str"/>
+      <x:c r="K105" s="34" t="str"/>
+      <x:c r="L105" s="34" t="str"/>
+      <x:c r="M105" s="36" t="str"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="46" t="str">
         <x:v>vermis</x:v>
       </x:c>
-      <x:c r="B105" s="39" t="str">
+      <x:c r="B106" s="39" t="str">
         <x:v>Vermis</x:v>
       </x:c>
-      <x:c r="C105" s="39" t="str">
-        <x:v>advanced</x:v>
-      </x:c>
-      <x:c r="D105" s="39" t="str">
+      <x:c r="C106" s="39" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="D106" s="39" t="str">
         <x:v>cerebellum; midline</x:v>
       </x:c>
-      <x:c r="E105" s="38" t="str"/>
-      <x:c r="F105" s="38" t="str"/>
-      <x:c r="G105" s="38" t="str"/>
-      <x:c r="H105" s="38" t="str"/>
-      <x:c r="I105" s="38" t="str"/>
-      <x:c r="J105" s="38" t="str"/>
-      <x:c r="K105" s="38" t="str"/>
-      <x:c r="L105" s="38" t="str"/>
-      <x:c r="M105" s="40" t="str"/>
+      <x:c r="E106" s="38" t="str"/>
+      <x:c r="F106" s="38" t="str"/>
+      <x:c r="G106" s="38" t="str"/>
+      <x:c r="H106" s="38" t="str"/>
+      <x:c r="I106" s="38" t="str"/>
+      <x:c r="J106" s="38" t="str"/>
+      <x:c r="K106" s="38" t="str"/>
+      <x:c r="L106" s="38" t="str"/>
+      <x:c r="M106" s="40" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8915a160bea24d4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f61e8b7eef648a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update accepted optic and callosal masks
</commit_message>
<xml_diff>
--- a/data/finalized/curation/brain_mri_curation.xlsx
+++ b/data/finalized/curation/brain_mri_curation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R362281277f0d48dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="R46e86ae690d14965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="R1e98051f2815417c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rec3e922869114c58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="R2255b6ad4e30435f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="Rdeb543391cdf452b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -375,7 +375,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StructureCurationTable" displayName="StructureCurationTable" ref="A1:L106" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StructureCurationTable" displayName="StructureCurationTable" ref="A1:L107" headerRowCount="1">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="include_in_viewer"/>
     <x:tableColumn id="2" name="difficulty"/>
@@ -395,7 +395,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuizQuestionTable" displayName="QuizQuestionTable" ref="A1:M106" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuizQuestionTable" displayName="QuizQuestionTable" ref="A1:M107" headerRowCount="1">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="display_name"/>
@@ -721,7 +721,7 @@
         <x:v>Structure count</x:v>
       </x:c>
       <x:c r="B9" s="5" t="n">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str"/>
       <x:c r="D9" s="5" t="str"/>
@@ -3343,32 +3343,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B89" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
-        <x:v>septum_pellucidum</x:v>
+        <x:v>rostrum_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>Septum pellucidum</x:v>
+        <x:v>Rostrum of the corpus callosum</x:v>
       </x:c>
       <x:c r="E89" s="35" t="str">
-        <x:v>midline; ventricles; csf_spaces</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F89" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G89" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H89" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I89" s="35" t="str">
-        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G89" s="35" t="str"/>
+      <x:c r="H89" s="35" t="str"/>
+      <x:c r="I89" s="35" t="str"/>
       <x:c r="J89" s="35" t="str"/>
       <x:c r="K89" s="35" t="str"/>
-      <x:c r="L89" s="36" t="str"/>
+      <x:c r="L89" s="36" t="str">
+        <x:v>Added from browser-created accepted mask; review in viewer/ITK-SNAP.</x:v>
+      </x:c>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="33" t="str">
@@ -3378,13 +3374,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
-        <x:v>splenium_of_the_corpus_callosum</x:v>
+        <x:v>septum_pellucidum</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>Splenium of the corpus callosum</x:v>
+        <x:v>Septum pellucidum</x:v>
       </x:c>
       <x:c r="E90" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F90" s="35" t="str">
         <x:v>yes</x:v>
@@ -3396,7 +3392,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I90" s="35" t="str">
-        <x:v>annotations/075_splenium_of_the_corpus_callosum.nii.gz</x:v>
+        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
       </x:c>
       <x:c r="J90" s="35" t="str"/>
       <x:c r="K90" s="35" t="str"/>
@@ -3410,57 +3406,57 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
-        <x:v>subthalamic_region</x:v>
+        <x:v>splenium_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>Subthalamic region</x:v>
+        <x:v>Splenium of the corpus callosum</x:v>
       </x:c>
       <x:c r="E91" s="35" t="str">
-        <x:v>deep_gray; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F91" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G91" s="35" t="str"/>
-      <x:c r="H91" s="35" t="str"/>
-      <x:c r="I91" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G91" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H91" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I91" s="35" t="str">
+        <x:v>annotations/075_splenium_of_the_corpus_callosum.nii.gz</x:v>
+      </x:c>
       <x:c r="J91" s="35" t="str"/>
       <x:c r="K91" s="35" t="str"/>
-      <x:c r="L91" s="36" t="str">
-        <x:v>Optional beginner-to-intermediate deep gray landmark if it can be shown cleanly on this T1.</x:v>
-      </x:c>
+      <x:c r="L91" s="36" t="str"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B92" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
-        <x:v>superior_frontal_gyrus</x:v>
+        <x:v>subthalamic_region</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>Superior frontal gyrus</x:v>
+        <x:v>Subthalamic region</x:v>
       </x:c>
       <x:c r="E92" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>deep_gray; basal_ganglia</x:v>
       </x:c>
       <x:c r="F92" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G92" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H92" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I92" s="35" t="str">
-        <x:v>annotations/024_superior_frontal_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G92" s="35" t="str"/>
+      <x:c r="H92" s="35" t="str"/>
+      <x:c r="I92" s="35" t="str"/>
       <x:c r="J92" s="35" t="str"/>
       <x:c r="K92" s="35" t="str"/>
-      <x:c r="L92" s="36" t="str"/>
+      <x:c r="L92" s="36" t="str">
+        <x:v>Optional beginner-to-intermediate deep gray landmark if it can be shown cleanly on this T1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="33" t="str">
@@ -3470,39 +3466,45 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
-        <x:v>superior_orbital_fissure</x:v>
+        <x:v>superior_frontal_gyrus</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>Superior orbital fissure</x:v>
+        <x:v>Superior frontal gyrus</x:v>
       </x:c>
       <x:c r="E93" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F93" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G93" s="35" t="str"/>
-      <x:c r="H93" s="35" t="str"/>
-      <x:c r="I93" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G93" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H93" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I93" s="35" t="str">
+        <x:v>annotations/024_superior_frontal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J93" s="35" t="str"/>
       <x:c r="K93" s="35" t="str"/>
       <x:c r="L93" s="36" t="str"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B94" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
-        <x:v>superior_temporal_gyrus</x:v>
+        <x:v>superior_orbital_fissure</x:v>
       </x:c>
       <x:c r="D94" s="35" t="str">
-        <x:v>Superior temporal gyrus</x:v>
+        <x:v>Superior orbital fissure</x:v>
       </x:c>
       <x:c r="E94" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="F94" s="35" t="str">
         <x:v>no</x:v>
@@ -3516,32 +3518,26 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B95" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C95" s="35" t="str">
-        <x:v>supramarginal_gyrus</x:v>
+        <x:v>superior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="D95" s="35" t="str">
-        <x:v>Supramarginal gyrus</x:v>
+        <x:v>Superior temporal gyrus</x:v>
       </x:c>
       <x:c r="E95" s="35" t="str">
         <x:v>cortex</x:v>
       </x:c>
       <x:c r="F95" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G95" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H95" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I95" s="35" t="str">
-        <x:v>annotations/025_supramarginal_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G95" s="35" t="str"/>
+      <x:c r="H95" s="35" t="str"/>
+      <x:c r="I95" s="35" t="str"/>
       <x:c r="J95" s="35" t="str"/>
       <x:c r="K95" s="35" t="str"/>
       <x:c r="L95" s="36" t="str"/>
@@ -3551,23 +3547,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B96" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C96" s="35" t="str">
-        <x:v>suprasellar_cistern</x:v>
+        <x:v>supramarginal_gyrus</x:v>
       </x:c>
       <x:c r="D96" s="35" t="str">
-        <x:v>Suprasellar cistern</x:v>
+        <x:v>Supramarginal gyrus</x:v>
       </x:c>
       <x:c r="E96" s="35" t="str">
-        <x:v>csf_spaces; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F96" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G96" s="35" t="str"/>
-      <x:c r="H96" s="35" t="str"/>
-      <x:c r="I96" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G96" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H96" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I96" s="35" t="str">
+        <x:v>annotations/025_supramarginal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J96" s="35" t="str"/>
       <x:c r="K96" s="35" t="str"/>
       <x:c r="L96" s="36" t="str"/>
@@ -3580,26 +3582,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C97" s="35" t="str">
-        <x:v>sylvian_fissure</x:v>
+        <x:v>suprasellar_cistern</x:v>
       </x:c>
       <x:c r="D97" s="35" t="str">
-        <x:v>Sylvian fissure</x:v>
+        <x:v>Suprasellar cistern</x:v>
       </x:c>
       <x:c r="E97" s="35" t="str">
-        <x:v>csf_spaces; cortex</x:v>
+        <x:v>csf_spaces; skull_base</x:v>
       </x:c>
       <x:c r="F97" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G97" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H97" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I97" s="35" t="str">
-        <x:v>annotations/051_sylvian_fissure.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G97" s="35" t="str"/>
+      <x:c r="H97" s="35" t="str"/>
+      <x:c r="I97" s="35" t="str"/>
       <x:c r="J97" s="35" t="str"/>
       <x:c r="K97" s="35" t="str"/>
       <x:c r="L97" s="36" t="str"/>
@@ -3612,13 +3608,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C98" s="35" t="str">
-        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>sylvian_fissure</x:v>
       </x:c>
       <x:c r="D98" s="35" t="str">
-        <x:v>Temporal horn of the lateral ventricle</x:v>
+        <x:v>Sylvian fissure</x:v>
       </x:c>
       <x:c r="E98" s="35" t="str">
-        <x:v>ventricles; csf_spaces; deep_gray</x:v>
+        <x:v>csf_spaces; cortex</x:v>
       </x:c>
       <x:c r="F98" s="35" t="str">
         <x:v>yes</x:v>
@@ -3630,7 +3626,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I98" s="35" t="str">
-        <x:v>annotations/045_temporal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/051_sylvian_fissure.nii.gz</x:v>
       </x:c>
       <x:c r="J98" s="35" t="str"/>
       <x:c r="K98" s="35" t="str"/>
@@ -3644,80 +3640,86 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C99" s="35" t="str">
-        <x:v>temporal_lobe</x:v>
+        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D99" s="35" t="str">
-        <x:v>Temporal lobe</x:v>
+        <x:v>Temporal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E99" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces; deep_gray</x:v>
       </x:c>
       <x:c r="F99" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G99" s="35" t="str"/>
-      <x:c r="H99" s="35" t="str"/>
-      <x:c r="I99" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G99" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H99" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I99" s="35" t="str">
+        <x:v>annotations/045_temporal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J99" s="35" t="str"/>
       <x:c r="K99" s="35" t="str"/>
-      <x:c r="L99" s="36" t="str">
-        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
-      </x:c>
+      <x:c r="L99" s="36" t="str"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B100" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C100" s="35" t="str">
-        <x:v>temporal_pole</x:v>
+        <x:v>temporal_lobe</x:v>
       </x:c>
       <x:c r="D100" s="35" t="str">
-        <x:v>Temporal pole</x:v>
+        <x:v>Temporal lobe</x:v>
       </x:c>
       <x:c r="E100" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="F100" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G100" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H100" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I100" s="35" t="str">
-        <x:v>annotations/026_temporal_pole.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G100" s="35" t="str"/>
+      <x:c r="H100" s="35" t="str"/>
+      <x:c r="I100" s="35" t="str"/>
       <x:c r="J100" s="35" t="str"/>
       <x:c r="K100" s="35" t="str"/>
-      <x:c r="L100" s="36" t="str"/>
+      <x:c r="L100" s="36" t="str">
+        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
+      </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B101" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C101" s="35" t="str">
-        <x:v>tentorium_cerebelli</x:v>
+        <x:v>temporal_pole</x:v>
       </x:c>
       <x:c r="D101" s="35" t="str">
-        <x:v>Tentorium cerebelli</x:v>
+        <x:v>Temporal pole</x:v>
       </x:c>
       <x:c r="E101" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F101" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G101" s="35" t="str"/>
-      <x:c r="H101" s="35" t="str"/>
-      <x:c r="I101" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G101" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H101" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I101" s="35" t="str">
+        <x:v>annotations/026_temporal_pole.nii.gz</x:v>
+      </x:c>
       <x:c r="J101" s="35" t="str"/>
       <x:c r="K101" s="35" t="str"/>
       <x:c r="L101" s="36" t="str"/>
@@ -3730,26 +3732,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C102" s="35" t="str">
-        <x:v>thalamus</x:v>
+        <x:v>tentorium_cerebelli</x:v>
       </x:c>
       <x:c r="D102" s="35" t="str">
-        <x:v>Thalamus</x:v>
+        <x:v>Tentorium cerebelli</x:v>
       </x:c>
       <x:c r="E102" s="35" t="str">
-        <x:v>deep_gray</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="F102" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G102" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H102" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I102" s="35" t="str">
-        <x:v>annotations/002_thalamus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G102" s="35" t="str"/>
+      <x:c r="H102" s="35" t="str"/>
+      <x:c r="I102" s="35" t="str"/>
       <x:c r="J102" s="35" t="str"/>
       <x:c r="K102" s="35" t="str"/>
       <x:c r="L102" s="36" t="str"/>
@@ -3762,13 +3758,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C103" s="35" t="str">
-        <x:v>third_ventricle</x:v>
+        <x:v>thalamus</x:v>
       </x:c>
       <x:c r="D103" s="35" t="str">
-        <x:v>Third ventricle</x:v>
+        <x:v>Thalamus</x:v>
       </x:c>
       <x:c r="E103" s="35" t="str">
-        <x:v>ventricles; csf_spaces; midline</x:v>
+        <x:v>deep_gray</x:v>
       </x:c>
       <x:c r="F103" s="35" t="str">
         <x:v>yes</x:v>
@@ -3780,7 +3776,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I103" s="35" t="str">
-        <x:v>annotations/006_third_ventricle.nii.gz</x:v>
+        <x:v>annotations/002_thalamus.nii.gz</x:v>
       </x:c>
       <x:c r="J103" s="35" t="str"/>
       <x:c r="K103" s="35" t="str"/>
@@ -3794,25 +3790,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C104" s="35" t="str">
-        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
+        <x:v>third_ventricle</x:v>
       </x:c>
       <x:c r="D104" s="35" t="str">
-        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
+        <x:v>Third ventricle</x:v>
       </x:c>
       <x:c r="E104" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; midline</x:v>
       </x:c>
       <x:c r="F104" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G104" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H104" s="35" t="str">
-        <x:v>accepted</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I104" s="35" t="str">
-        <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/006_third_ventricle.nii.gz</x:v>
       </x:c>
       <x:c r="J104" s="35" t="str"/>
       <x:c r="K104" s="35" t="str"/>
@@ -3823,65 +3819,97 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B105" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C105" s="35" t="str">
-        <x:v>uncus</x:v>
+        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D105" s="35" t="str">
-        <x:v>Uncus</x:v>
+        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E105" s="35" t="str">
-        <x:v>limbic; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F105" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G105" s="35" t="str"/>
-      <x:c r="H105" s="35" t="str"/>
-      <x:c r="I105" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G105" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H105" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I105" s="35" t="str">
+        <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J105" s="35" t="str"/>
       <x:c r="K105" s="35" t="str"/>
       <x:c r="L105" s="36" t="str"/>
     </x:row>
     <x:row r="106">
-      <x:c r="A106" s="37" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="B106" s="38" t="str">
-        <x:v>advanced</x:v>
-      </x:c>
-      <x:c r="C106" s="39" t="str">
+      <x:c r="A106" s="33" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="B106" s="34" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="C106" s="35" t="str">
+        <x:v>uncus</x:v>
+      </x:c>
+      <x:c r="D106" s="35" t="str">
+        <x:v>Uncus</x:v>
+      </x:c>
+      <x:c r="E106" s="35" t="str">
+        <x:v>limbic; cortex</x:v>
+      </x:c>
+      <x:c r="F106" s="35" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G106" s="35" t="str"/>
+      <x:c r="H106" s="35" t="str"/>
+      <x:c r="I106" s="35" t="str"/>
+      <x:c r="J106" s="35" t="str"/>
+      <x:c r="K106" s="35" t="str"/>
+      <x:c r="L106" s="36" t="str"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="37" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="B107" s="38" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="C107" s="39" t="str">
         <x:v>vermis</x:v>
       </x:c>
-      <x:c r="D106" s="39" t="str">
+      <x:c r="D107" s="39" t="str">
         <x:v>Vermis</x:v>
       </x:c>
-      <x:c r="E106" s="39" t="str">
+      <x:c r="E107" s="39" t="str">
         <x:v>cerebellum; midline</x:v>
       </x:c>
-      <x:c r="F106" s="39" t="str">
+      <x:c r="F107" s="39" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="G106" s="39" t="str"/>
-      <x:c r="H106" s="39" t="str"/>
-      <x:c r="I106" s="39" t="str"/>
-      <x:c r="J106" s="39" t="str"/>
-      <x:c r="K106" s="39" t="str"/>
-      <x:c r="L106" s="40" t="str"/>
+      <x:c r="G107" s="39" t="str"/>
+      <x:c r="H107" s="39" t="str"/>
+      <x:c r="I107" s="39" t="str"/>
+      <x:c r="J107" s="39" t="str"/>
+      <x:c r="K107" s="39" t="str"/>
+      <x:c r="L107" s="40" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="A2:A106">
+    <x:dataValidation type="list" sqref="A2:A107">
       <x:formula1>"yes,no"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="B2:B106">
+    <x:dataValidation type="list" sqref="B2:B107">
       <x:formula1>"beginner,advanced"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6edf86a302a14020"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30dc6bc66f7c4a6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5949,16 +5977,16 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="45" t="str">
-        <x:v>septum_pellucidum</x:v>
+        <x:v>rostrum_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="B89" s="35" t="str">
-        <x:v>Septum pellucidum</x:v>
+        <x:v>Rostrum of the corpus callosum</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>midline; ventricles; csf_spaces</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E89" s="34" t="str"/>
       <x:c r="F89" s="34" t="str"/>
@@ -5972,16 +6000,16 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="45" t="str">
-        <x:v>splenium_of_the_corpus_callosum</x:v>
+        <x:v>septum_pellucidum</x:v>
       </x:c>
       <x:c r="B90" s="35" t="str">
-        <x:v>Splenium of the corpus callosum</x:v>
+        <x:v>Septum pellucidum</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E90" s="34" t="str"/>
       <x:c r="F90" s="34" t="str"/>
@@ -5995,16 +6023,16 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="45" t="str">
-        <x:v>subthalamic_region</x:v>
+        <x:v>splenium_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="B91" s="35" t="str">
-        <x:v>Subthalamic region</x:v>
+        <x:v>Splenium of the corpus callosum</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>deep_gray; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E91" s="34" t="str"/>
       <x:c r="F91" s="34" t="str"/>
@@ -6018,16 +6046,16 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="45" t="str">
-        <x:v>superior_frontal_gyrus</x:v>
+        <x:v>subthalamic_region</x:v>
       </x:c>
       <x:c r="B92" s="35" t="str">
-        <x:v>Superior frontal gyrus</x:v>
+        <x:v>Subthalamic region</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>deep_gray; basal_ganglia</x:v>
       </x:c>
       <x:c r="E92" s="34" t="str"/>
       <x:c r="F92" s="34" t="str"/>
@@ -6041,16 +6069,16 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="45" t="str">
-        <x:v>superior_orbital_fissure</x:v>
+        <x:v>superior_frontal_gyrus</x:v>
       </x:c>
       <x:c r="B93" s="35" t="str">
-        <x:v>Superior orbital fissure</x:v>
+        <x:v>Superior frontal gyrus</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E93" s="34" t="str"/>
       <x:c r="F93" s="34" t="str"/>
@@ -6064,16 +6092,16 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="45" t="str">
-        <x:v>superior_temporal_gyrus</x:v>
+        <x:v>superior_orbital_fissure</x:v>
       </x:c>
       <x:c r="B94" s="35" t="str">
-        <x:v>Superior temporal gyrus</x:v>
+        <x:v>Superior orbital fissure</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D94" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="E94" s="34" t="str"/>
       <x:c r="F94" s="34" t="str"/>
@@ -6087,13 +6115,13 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="45" t="str">
-        <x:v>supramarginal_gyrus</x:v>
+        <x:v>superior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="B95" s="35" t="str">
-        <x:v>Supramarginal gyrus</x:v>
+        <x:v>Superior temporal gyrus</x:v>
       </x:c>
       <x:c r="C95" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D95" s="35" t="str">
         <x:v>cortex</x:v>
@@ -6110,16 +6138,16 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="45" t="str">
-        <x:v>suprasellar_cistern</x:v>
+        <x:v>supramarginal_gyrus</x:v>
       </x:c>
       <x:c r="B96" s="35" t="str">
-        <x:v>Suprasellar cistern</x:v>
+        <x:v>Supramarginal gyrus</x:v>
       </x:c>
       <x:c r="C96" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D96" s="35" t="str">
-        <x:v>csf_spaces; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E96" s="34" t="str"/>
       <x:c r="F96" s="34" t="str"/>
@@ -6133,16 +6161,16 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="45" t="str">
-        <x:v>sylvian_fissure</x:v>
+        <x:v>suprasellar_cistern</x:v>
       </x:c>
       <x:c r="B97" s="35" t="str">
-        <x:v>Sylvian fissure</x:v>
+        <x:v>Suprasellar cistern</x:v>
       </x:c>
       <x:c r="C97" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D97" s="35" t="str">
-        <x:v>csf_spaces; cortex</x:v>
+        <x:v>csf_spaces; skull_base</x:v>
       </x:c>
       <x:c r="E97" s="34" t="str"/>
       <x:c r="F97" s="34" t="str"/>
@@ -6156,16 +6184,16 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="45" t="str">
-        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>sylvian_fissure</x:v>
       </x:c>
       <x:c r="B98" s="35" t="str">
-        <x:v>Temporal horn of the lateral ventricle</x:v>
+        <x:v>Sylvian fissure</x:v>
       </x:c>
       <x:c r="C98" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D98" s="35" t="str">
-        <x:v>ventricles; csf_spaces; deep_gray</x:v>
+        <x:v>csf_spaces; cortex</x:v>
       </x:c>
       <x:c r="E98" s="34" t="str"/>
       <x:c r="F98" s="34" t="str"/>
@@ -6179,16 +6207,16 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="45" t="str">
-        <x:v>temporal_lobe</x:v>
+        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B99" s="35" t="str">
-        <x:v>Temporal lobe</x:v>
+        <x:v>Temporal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C99" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D99" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces; deep_gray</x:v>
       </x:c>
       <x:c r="E99" s="34" t="str"/>
       <x:c r="F99" s="34" t="str"/>
@@ -6202,16 +6230,16 @@
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="45" t="str">
-        <x:v>temporal_pole</x:v>
+        <x:v>temporal_lobe</x:v>
       </x:c>
       <x:c r="B100" s="35" t="str">
-        <x:v>Temporal pole</x:v>
+        <x:v>Temporal lobe</x:v>
       </x:c>
       <x:c r="C100" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D100" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="E100" s="34" t="str"/>
       <x:c r="F100" s="34" t="str"/>
@@ -6225,16 +6253,16 @@
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="45" t="str">
-        <x:v>tentorium_cerebelli</x:v>
+        <x:v>temporal_pole</x:v>
       </x:c>
       <x:c r="B101" s="35" t="str">
-        <x:v>Tentorium cerebelli</x:v>
+        <x:v>Temporal pole</x:v>
       </x:c>
       <x:c r="C101" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D101" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E101" s="34" t="str"/>
       <x:c r="F101" s="34" t="str"/>
@@ -6248,16 +6276,16 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="45" t="str">
-        <x:v>thalamus</x:v>
+        <x:v>tentorium_cerebelli</x:v>
       </x:c>
       <x:c r="B102" s="35" t="str">
-        <x:v>Thalamus</x:v>
+        <x:v>Tentorium cerebelli</x:v>
       </x:c>
       <x:c r="C102" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D102" s="35" t="str">
-        <x:v>deep_gray</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="E102" s="34" t="str"/>
       <x:c r="F102" s="34" t="str"/>
@@ -6271,16 +6299,16 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="45" t="str">
-        <x:v>third_ventricle</x:v>
+        <x:v>thalamus</x:v>
       </x:c>
       <x:c r="B103" s="35" t="str">
-        <x:v>Third ventricle</x:v>
+        <x:v>Thalamus</x:v>
       </x:c>
       <x:c r="C103" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D103" s="35" t="str">
-        <x:v>ventricles; csf_spaces; midline</x:v>
+        <x:v>deep_gray</x:v>
       </x:c>
       <x:c r="E103" s="34" t="str"/>
       <x:c r="F103" s="34" t="str"/>
@@ -6294,16 +6322,16 @@
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="45" t="str">
-        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
+        <x:v>third_ventricle</x:v>
       </x:c>
       <x:c r="B104" s="35" t="str">
-        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
+        <x:v>Third ventricle</x:v>
       </x:c>
       <x:c r="C104" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D104" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; midline</x:v>
       </x:c>
       <x:c r="E104" s="34" t="str"/>
       <x:c r="F104" s="34" t="str"/>
@@ -6317,16 +6345,16 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="45" t="str">
-        <x:v>uncus</x:v>
+        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B105" s="35" t="str">
-        <x:v>Uncus</x:v>
+        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C105" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D105" s="35" t="str">
-        <x:v>limbic; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E105" s="34" t="str"/>
       <x:c r="F105" s="34" t="str"/>
@@ -6339,32 +6367,55 @@
       <x:c r="M105" s="36" t="str"/>
     </x:row>
     <x:row r="106">
-      <x:c r="A106" s="46" t="str">
+      <x:c r="A106" s="45" t="str">
+        <x:v>uncus</x:v>
+      </x:c>
+      <x:c r="B106" s="35" t="str">
+        <x:v>Uncus</x:v>
+      </x:c>
+      <x:c r="C106" s="35" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="D106" s="35" t="str">
+        <x:v>limbic; cortex</x:v>
+      </x:c>
+      <x:c r="E106" s="34" t="str"/>
+      <x:c r="F106" s="34" t="str"/>
+      <x:c r="G106" s="34" t="str"/>
+      <x:c r="H106" s="34" t="str"/>
+      <x:c r="I106" s="34" t="str"/>
+      <x:c r="J106" s="34" t="str"/>
+      <x:c r="K106" s="34" t="str"/>
+      <x:c r="L106" s="34" t="str"/>
+      <x:c r="M106" s="36" t="str"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="46" t="str">
         <x:v>vermis</x:v>
       </x:c>
-      <x:c r="B106" s="39" t="str">
+      <x:c r="B107" s="39" t="str">
         <x:v>Vermis</x:v>
       </x:c>
-      <x:c r="C106" s="39" t="str">
-        <x:v>advanced</x:v>
-      </x:c>
-      <x:c r="D106" s="39" t="str">
+      <x:c r="C107" s="39" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="D107" s="39" t="str">
         <x:v>cerebellum; midline</x:v>
       </x:c>
-      <x:c r="E106" s="38" t="str"/>
-      <x:c r="F106" s="38" t="str"/>
-      <x:c r="G106" s="38" t="str"/>
-      <x:c r="H106" s="38" t="str"/>
-      <x:c r="I106" s="38" t="str"/>
-      <x:c r="J106" s="38" t="str"/>
-      <x:c r="K106" s="38" t="str"/>
-      <x:c r="L106" s="38" t="str"/>
-      <x:c r="M106" s="40" t="str"/>
+      <x:c r="E107" s="38" t="str"/>
+      <x:c r="F107" s="38" t="str"/>
+      <x:c r="G107" s="38" t="str"/>
+      <x:c r="H107" s="38" t="str"/>
+      <x:c r="I107" s="38" t="str"/>
+      <x:c r="J107" s="38" t="str"/>
+      <x:c r="K107" s="38" t="str"/>
+      <x:c r="L107" s="38" t="str"/>
+      <x:c r="M107" s="40" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f61e8b7eef648a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39c52bf375db4545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add combined corpus callosum mask
</commit_message>
<xml_diff>
--- a/data/finalized/curation/brain_mri_curation.xlsx
+++ b/data/finalized/curation/brain_mri_curation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rec3e922869114c58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="R2255b6ad4e30435f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="Rdeb543391cdf452b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R14949da8a8db4248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="Rd337bb02575a4ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="Re6d25cd770dd46b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -375,7 +375,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StructureCurationTable" displayName="StructureCurationTable" ref="A1:L107" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StructureCurationTable" displayName="StructureCurationTable" ref="A1:L108" headerRowCount="1">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="include_in_viewer"/>
     <x:tableColumn id="2" name="difficulty"/>
@@ -395,7 +395,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuizQuestionTable" displayName="QuizQuestionTable" ref="A1:M107" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuizQuestionTable" displayName="QuizQuestionTable" ref="A1:M108" headerRowCount="1">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="display_name"/>
@@ -721,7 +721,7 @@
         <x:v>Structure count</x:v>
       </x:c>
       <x:c r="B9" s="5" t="n">
-        <x:v>106</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str"/>
       <x:c r="D9" s="5" t="str"/>
@@ -1440,52 +1440,54 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C24" s="35" t="str">
-        <x:v>crista_galli</x:v>
+        <x:v>corpus_callosum</x:v>
       </x:c>
       <x:c r="D24" s="35" t="str">
-        <x:v>Crista galli</x:v>
+        <x:v>Corpus callosum</x:v>
       </x:c>
       <x:c r="E24" s="35" t="str">
-        <x:v>skull_base; midline</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F24" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G24" s="35" t="str"/>
-      <x:c r="H24" s="35" t="str"/>
-      <x:c r="I24" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G24" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H24" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I24" s="35" t="str">
+        <x:v>annotations/107_corpus_callosum.nii.gz</x:v>
+      </x:c>
       <x:c r="J24" s="35" t="str"/>
       <x:c r="K24" s="35" t="str"/>
-      <x:c r="L24" s="36" t="str"/>
+      <x:c r="L24" s="36" t="str">
+        <x:v>Composite union of rostrum, genu, body, and splenium masks.</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B25" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C25" s="35" t="str">
-        <x:v>cuneus</x:v>
+        <x:v>crista_galli</x:v>
       </x:c>
       <x:c r="D25" s="35" t="str">
-        <x:v>Cuneus</x:v>
+        <x:v>Crista galli</x:v>
       </x:c>
       <x:c r="E25" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; midline</x:v>
       </x:c>
       <x:c r="F25" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G25" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H25" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I25" s="35" t="str">
-        <x:v>annotations/013_cuneus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G25" s="35" t="str"/>
+      <x:c r="H25" s="35" t="str"/>
+      <x:c r="I25" s="35" t="str"/>
       <x:c r="J25" s="35" t="str"/>
       <x:c r="K25" s="35" t="str"/>
       <x:c r="L25" s="36" t="str"/>
@@ -1498,25 +1500,25 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C26" s="35" t="str">
-        <x:v>entorhinal_cortex</x:v>
+        <x:v>cuneus</x:v>
       </x:c>
       <x:c r="D26" s="35" t="str">
-        <x:v>Entorhinal cortex</x:v>
+        <x:v>Cuneus</x:v>
       </x:c>
       <x:c r="E26" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F26" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G26" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H26" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I26" s="35" t="str">
-        <x:v>annotations/014_entorhinal_cortex.nii.gz</x:v>
+        <x:v>annotations/013_cuneus.nii.gz</x:v>
       </x:c>
       <x:c r="J26" s="35" t="str"/>
       <x:c r="K26" s="35" t="str"/>
@@ -1527,23 +1529,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B27" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C27" s="35" t="str">
-        <x:v>external_auditory_canal</x:v>
+        <x:v>entorhinal_cortex</x:v>
       </x:c>
       <x:c r="D27" s="35" t="str">
-        <x:v>External auditory canal</x:v>
+        <x:v>Entorhinal cortex</x:v>
       </x:c>
       <x:c r="E27" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="F27" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G27" s="35" t="str"/>
-      <x:c r="H27" s="35" t="str"/>
-      <x:c r="I27" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G27" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H27" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I27" s="35" t="str">
+        <x:v>annotations/014_entorhinal_cortex.nii.gz</x:v>
+      </x:c>
       <x:c r="J27" s="35" t="str"/>
       <x:c r="K27" s="35" t="str"/>
       <x:c r="L27" s="36" t="str"/>
@@ -1556,13 +1564,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C28" s="35" t="str">
-        <x:v>falx_cerebri</x:v>
+        <x:v>external_auditory_canal</x:v>
       </x:c>
       <x:c r="D28" s="35" t="str">
-        <x:v>Falx cerebri</x:v>
+        <x:v>External auditory canal</x:v>
       </x:c>
       <x:c r="E28" s="35" t="str">
-        <x:v>midline</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="F28" s="35" t="str">
         <x:v>no</x:v>
@@ -1582,13 +1590,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C29" s="35" t="str">
-        <x:v>foramen_magnum</x:v>
+        <x:v>falx_cerebri</x:v>
       </x:c>
       <x:c r="D29" s="35" t="str">
-        <x:v>Foramen magnum</x:v>
+        <x:v>Falx cerebri</x:v>
       </x:c>
       <x:c r="E29" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>midline</x:v>
       </x:c>
       <x:c r="F29" s="35" t="str">
         <x:v>no</x:v>
@@ -1602,19 +1610,19 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B30" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C30" s="35" t="str">
-        <x:v>foramen_of_luschka</x:v>
+        <x:v>foramen_magnum</x:v>
       </x:c>
       <x:c r="D30" s="35" t="str">
-        <x:v>Foramen of Luschka</x:v>
+        <x:v>Foramen magnum</x:v>
       </x:c>
       <x:c r="E30" s="35" t="str">
-        <x:v>ventricles; csf_spaces; brainstem</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="F30" s="35" t="str">
         <x:v>no</x:v>
@@ -1634,10 +1642,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C31" s="35" t="str">
-        <x:v>foramen_of_magendie</x:v>
+        <x:v>foramen_of_luschka</x:v>
       </x:c>
       <x:c r="D31" s="35" t="str">
-        <x:v>Foramen of Magendie</x:v>
+        <x:v>Foramen of Luschka</x:v>
       </x:c>
       <x:c r="E31" s="35" t="str">
         <x:v>ventricles; csf_spaces; brainstem</x:v>
@@ -1654,32 +1662,26 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B32" s="34" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C32" s="35" t="str">
-        <x:v>forceps_major</x:v>
+        <x:v>foramen_of_magendie</x:v>
       </x:c>
       <x:c r="D32" s="35" t="str">
-        <x:v>Forceps major</x:v>
+        <x:v>Foramen of Magendie</x:v>
       </x:c>
       <x:c r="E32" s="35" t="str">
-        <x:v>white_matter</x:v>
+        <x:v>ventricles; csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F32" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G32" s="35" t="str">
-        <x:v>rough_support</x:v>
-      </x:c>
-      <x:c r="H32" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I32" s="35" t="str">
-        <x:v>annotations/078_forceps_major.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G32" s="35" t="str"/>
+      <x:c r="H32" s="35" t="str"/>
+      <x:c r="I32" s="35" t="str"/>
       <x:c r="J32" s="35" t="str"/>
       <x:c r="K32" s="35" t="str"/>
       <x:c r="L32" s="36" t="str"/>
@@ -1692,10 +1694,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C33" s="35" t="str">
-        <x:v>forceps_minor</x:v>
+        <x:v>forceps_major</x:v>
       </x:c>
       <x:c r="D33" s="35" t="str">
-        <x:v>Forceps minor</x:v>
+        <x:v>Forceps major</x:v>
       </x:c>
       <x:c r="E33" s="35" t="str">
         <x:v>white_matter</x:v>
@@ -1710,7 +1712,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I33" s="35" t="str">
-        <x:v>annotations/072_forceps_minor.nii.gz</x:v>
+        <x:v>annotations/078_forceps_major.nii.gz</x:v>
       </x:c>
       <x:c r="J33" s="35" t="str"/>
       <x:c r="K33" s="35" t="str"/>
@@ -1721,28 +1723,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B34" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C34" s="35" t="str">
-        <x:v>fourth_ventricle</x:v>
+        <x:v>forceps_minor</x:v>
       </x:c>
       <x:c r="D34" s="35" t="str">
-        <x:v>Fourth ventricle</x:v>
+        <x:v>Forceps minor</x:v>
       </x:c>
       <x:c r="E34" s="35" t="str">
-        <x:v>ventricles; csf_spaces; brainstem</x:v>
+        <x:v>white_matter</x:v>
       </x:c>
       <x:c r="F34" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G34" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
+        <x:v>rough_support</x:v>
       </x:c>
       <x:c r="H34" s="35" t="str">
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I34" s="35" t="str">
-        <x:v>annotations/007_fourth_ventricle.nii.gz</x:v>
+        <x:v>annotations/072_forceps_minor.nii.gz</x:v>
       </x:c>
       <x:c r="J34" s="35" t="str"/>
       <x:c r="K34" s="35" t="str"/>
@@ -1756,25 +1758,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C35" s="35" t="str">
-        <x:v>frontal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>fourth_ventricle</x:v>
       </x:c>
       <x:c r="D35" s="35" t="str">
-        <x:v>Frontal horn of the lateral ventricle</x:v>
+        <x:v>Fourth ventricle</x:v>
       </x:c>
       <x:c r="E35" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F35" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G35" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H35" s="35" t="str">
-        <x:v>accepted</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I35" s="35" t="str">
-        <x:v>annotations/061_frontal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/007_fourth_ventricle.nii.gz</x:v>
       </x:c>
       <x:c r="J35" s="35" t="str"/>
       <x:c r="K35" s="35" t="str"/>
@@ -1788,85 +1790,85 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C36" s="35" t="str">
-        <x:v>frontal_lobe</x:v>
+        <x:v>frontal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D36" s="35" t="str">
-        <x:v>Frontal lobe</x:v>
+        <x:v>Frontal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E36" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F36" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G36" s="35" t="str"/>
-      <x:c r="H36" s="35" t="str"/>
-      <x:c r="I36" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G36" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H36" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I36" s="35" t="str">
+        <x:v>annotations/061_frontal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J36" s="35" t="str"/>
       <x:c r="K36" s="35" t="str"/>
-      <x:c r="L36" s="36" t="str">
-        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
-      </x:c>
+      <x:c r="L36" s="36" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B37" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C37" s="35" t="str">
-        <x:v>fusiform_gyrus</x:v>
+        <x:v>frontal_lobe</x:v>
       </x:c>
       <x:c r="D37" s="35" t="str">
-        <x:v>Fusiform gyrus</x:v>
+        <x:v>Frontal lobe</x:v>
       </x:c>
       <x:c r="E37" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="F37" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G37" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H37" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I37" s="35" t="str">
-        <x:v>annotations/015_fusiform_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G37" s="35" t="str"/>
+      <x:c r="H37" s="35" t="str"/>
+      <x:c r="I37" s="35" t="str"/>
       <x:c r="J37" s="35" t="str"/>
       <x:c r="K37" s="35" t="str"/>
-      <x:c r="L37" s="36" t="str"/>
+      <x:c r="L37" s="36" t="str">
+        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B38" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C38" s="35" t="str">
-        <x:v>genu_of_the_corpus_callosum</x:v>
+        <x:v>fusiform_gyrus</x:v>
       </x:c>
       <x:c r="D38" s="35" t="str">
-        <x:v>Genu of the corpus callosum</x:v>
+        <x:v>Fusiform gyrus</x:v>
       </x:c>
       <x:c r="E38" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F38" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G38" s="35" t="str">
-        <x:v>rough_support</x:v>
+        <x:v>full_gyrus_composite</x:v>
       </x:c>
       <x:c r="H38" s="35" t="str">
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I38" s="35" t="str">
-        <x:v>annotations/060_genu_of_the_corpus_callosum.nii.gz</x:v>
+        <x:v>annotations/015_fusiform_gyrus.nii.gz</x:v>
       </x:c>
       <x:c r="J38" s="35" t="str"/>
       <x:c r="K38" s="35" t="str"/>
@@ -1877,23 +1879,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B39" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C39" s="35" t="str">
-        <x:v>genu_of_the_internal_capsule</x:v>
+        <x:v>genu_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="D39" s="35" t="str">
-        <x:v>Genu of the internal capsule</x:v>
+        <x:v>Genu of the corpus callosum</x:v>
       </x:c>
       <x:c r="E39" s="35" t="str">
-        <x:v>white_matter; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F39" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G39" s="35" t="str"/>
-      <x:c r="H39" s="35" t="str"/>
-      <x:c r="I39" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G39" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H39" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I39" s="35" t="str">
+        <x:v>annotations/060_genu_of_the_corpus_callosum.nii.gz</x:v>
+      </x:c>
       <x:c r="J39" s="35" t="str"/>
       <x:c r="K39" s="35" t="str"/>
       <x:c r="L39" s="36" t="str"/>
@@ -1903,29 +1911,23 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B40" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C40" s="35" t="str">
-        <x:v>globus_pallidus</x:v>
+        <x:v>genu_of_the_internal_capsule</x:v>
       </x:c>
       <x:c r="D40" s="35" t="str">
-        <x:v>Globus pallidus</x:v>
+        <x:v>Genu of the internal capsule</x:v>
       </x:c>
       <x:c r="E40" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>white_matter; basal_ganglia</x:v>
       </x:c>
       <x:c r="F40" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G40" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H40" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I40" s="35" t="str">
-        <x:v>annotations/005_globus_pallidus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G40" s="35" t="str"/>
+      <x:c r="H40" s="35" t="str"/>
+      <x:c r="I40" s="35" t="str"/>
       <x:c r="J40" s="35" t="str"/>
       <x:c r="K40" s="35" t="str"/>
       <x:c r="L40" s="36" t="str"/>
@@ -1935,28 +1937,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B41" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C41" s="35" t="str">
-        <x:v>gyrus_rectus</x:v>
+        <x:v>globus_pallidus</x:v>
       </x:c>
       <x:c r="D41" s="35" t="str">
-        <x:v>Gyrus rectus</x:v>
+        <x:v>Globus pallidus</x:v>
       </x:c>
       <x:c r="E41" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="F41" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G41" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H41" s="35" t="str">
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I41" s="35" t="str">
-        <x:v>annotations/041_gyrus_rectus.nii.gz</x:v>
+        <x:v>annotations/005_globus_pallidus.nii.gz</x:v>
       </x:c>
       <x:c r="J41" s="35" t="str"/>
       <x:c r="K41" s="35" t="str"/>
@@ -1967,44 +1969,48 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B42" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C42" s="35" t="str">
-        <x:v>habenula</x:v>
+        <x:v>gyrus_rectus</x:v>
       </x:c>
       <x:c r="D42" s="35" t="str">
-        <x:v>Habenula</x:v>
+        <x:v>Gyrus rectus</x:v>
       </x:c>
       <x:c r="E42" s="35" t="str">
-        <x:v>midline; deep_gray</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F42" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G42" s="35" t="str"/>
-      <x:c r="H42" s="35" t="str"/>
-      <x:c r="I42" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G42" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H42" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I42" s="35" t="str">
+        <x:v>annotations/041_gyrus_rectus.nii.gz</x:v>
+      </x:c>
       <x:c r="J42" s="35" t="str"/>
       <x:c r="K42" s="35" t="str"/>
-      <x:c r="L42" s="36" t="str">
-        <x:v>Small pineal/posterior commissural region landmark; include if visible enough for teaching.</x:v>
-      </x:c>
+      <x:c r="L42" s="36" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B43" s="34" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C43" s="35" t="str">
-        <x:v>hand_bump_of_the_precentral_gyrus</x:v>
+        <x:v>habenula</x:v>
       </x:c>
       <x:c r="D43" s="35" t="str">
-        <x:v>Hand bump of the precentral gyrus</x:v>
+        <x:v>Habenula</x:v>
       </x:c>
       <x:c r="E43" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>midline; deep_gray</x:v>
       </x:c>
       <x:c r="F43" s="35" t="str">
         <x:v>no</x:v>
@@ -2014,23 +2020,25 @@
       <x:c r="I43" s="35" t="str"/>
       <x:c r="J43" s="35" t="str"/>
       <x:c r="K43" s="35" t="str"/>
-      <x:c r="L43" s="36" t="str"/>
+      <x:c r="L43" s="36" t="str">
+        <x:v>Small pineal/posterior commissural region landmark; include if visible enough for teaching.</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B44" s="34" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C44" s="35" t="str">
-        <x:v>head_of_the_caudate_nucleus</x:v>
+        <x:v>hand_bump_of_the_precentral_gyrus</x:v>
       </x:c>
       <x:c r="D44" s="35" t="str">
-        <x:v>Head of the caudate nucleus</x:v>
+        <x:v>Hand bump of the precentral gyrus</x:v>
       </x:c>
       <x:c r="E44" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F44" s="35" t="str">
         <x:v>no</x:v>
@@ -2050,26 +2058,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C45" s="35" t="str">
-        <x:v>hippocampus</x:v>
+        <x:v>head_of_the_caudate_nucleus</x:v>
       </x:c>
       <x:c r="D45" s="35" t="str">
-        <x:v>Hippocampus</x:v>
+        <x:v>Head of the caudate nucleus</x:v>
       </x:c>
       <x:c r="E45" s="35" t="str">
-        <x:v>limbic</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="F45" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G45" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H45" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I45" s="35" t="str">
-        <x:v>annotations/008_hippocampus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G45" s="35" t="str"/>
+      <x:c r="H45" s="35" t="str"/>
+      <x:c r="I45" s="35" t="str"/>
       <x:c r="J45" s="35" t="str"/>
       <x:c r="K45" s="35" t="str"/>
       <x:c r="L45" s="36" t="str"/>
@@ -2079,42 +2081,48 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B46" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C46" s="35" t="str">
-        <x:v>inferior_colliculus</x:v>
+        <x:v>hippocampus</x:v>
       </x:c>
       <x:c r="D46" s="35" t="str">
-        <x:v>Inferior colliculus</x:v>
+        <x:v>Hippocampus</x:v>
       </x:c>
       <x:c r="E46" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>limbic</x:v>
       </x:c>
       <x:c r="F46" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G46" s="35" t="str"/>
-      <x:c r="H46" s="35" t="str"/>
-      <x:c r="I46" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G46" s="35" t="str">
+        <x:v>freesurfer_seed_split</x:v>
+      </x:c>
+      <x:c r="H46" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I46" s="35" t="str">
+        <x:v>annotations/008_hippocampus.nii.gz</x:v>
+      </x:c>
       <x:c r="J46" s="35" t="str"/>
       <x:c r="K46" s="35" t="str"/>
       <x:c r="L46" s="36" t="str"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B47" s="34" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C47" s="35" t="str">
-        <x:v>inferior_temporal_gyrus</x:v>
+        <x:v>inferior_colliculus</x:v>
       </x:c>
       <x:c r="D47" s="35" t="str">
-        <x:v>Inferior temporal gyrus</x:v>
+        <x:v>Inferior colliculus</x:v>
       </x:c>
       <x:c r="E47" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="F47" s="35" t="str">
         <x:v>no</x:v>
@@ -2128,32 +2136,26 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B48" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C48" s="35" t="str">
-        <x:v>insular_cortex</x:v>
+        <x:v>inferior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="D48" s="35" t="str">
-        <x:v>Insular cortex</x:v>
+        <x:v>Inferior temporal gyrus</x:v>
       </x:c>
       <x:c r="E48" s="35" t="str">
         <x:v>cortex</x:v>
       </x:c>
       <x:c r="F48" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G48" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H48" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I48" s="35" t="str">
-        <x:v>annotations/027_insular_cortex.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G48" s="35" t="str"/>
+      <x:c r="H48" s="35" t="str"/>
+      <x:c r="I48" s="35" t="str"/>
       <x:c r="J48" s="35" t="str"/>
       <x:c r="K48" s="35" t="str"/>
       <x:c r="L48" s="36" t="str"/>
@@ -2166,25 +2168,29 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C49" s="35" t="str">
-        <x:v>internal_auditory_canal</x:v>
+        <x:v>insular_cortex</x:v>
       </x:c>
       <x:c r="D49" s="35" t="str">
-        <x:v>Internal auditory canal</x:v>
+        <x:v>Insular cortex</x:v>
       </x:c>
       <x:c r="E49" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F49" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G49" s="35" t="str"/>
-      <x:c r="H49" s="35" t="str"/>
-      <x:c r="I49" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G49" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H49" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I49" s="35" t="str">
+        <x:v>annotations/027_insular_cortex.nii.gz</x:v>
+      </x:c>
       <x:c r="J49" s="35" t="str"/>
       <x:c r="K49" s="35" t="str"/>
-      <x:c r="L49" s="36" t="str">
-        <x:v>High-yield skull base landmark; useful before adding detailed foraminal contents questions.</x:v>
-      </x:c>
+      <x:c r="L49" s="36" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="33" t="str">
@@ -2194,13 +2200,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C50" s="35" t="str">
-        <x:v>interpeduncular_cistern</x:v>
+        <x:v>internal_auditory_canal</x:v>
       </x:c>
       <x:c r="D50" s="35" t="str">
-        <x:v>Interpeduncular cistern</x:v>
+        <x:v>Internal auditory canal</x:v>
       </x:c>
       <x:c r="E50" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="F50" s="35" t="str">
         <x:v>no</x:v>
@@ -2210,7 +2216,9 @@
       <x:c r="I50" s="35" t="str"/>
       <x:c r="J50" s="35" t="str"/>
       <x:c r="K50" s="35" t="str"/>
-      <x:c r="L50" s="36" t="str"/>
+      <x:c r="L50" s="36" t="str">
+        <x:v>High-yield skull base landmark; useful before adding detailed foraminal contents questions.</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="33" t="str">
@@ -2220,13 +2228,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C51" s="35" t="str">
-        <x:v>interventricular_foramen_foramen_of_monro</x:v>
+        <x:v>interpeduncular_cistern</x:v>
       </x:c>
       <x:c r="D51" s="35" t="str">
-        <x:v>Interventricular foramen (foramen of Monro)</x:v>
+        <x:v>Interpeduncular cistern</x:v>
       </x:c>
       <x:c r="E51" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F51" s="35" t="str">
         <x:v>no</x:v>
@@ -2236,9 +2244,7 @@
       <x:c r="I51" s="35" t="str"/>
       <x:c r="J51" s="35" t="str"/>
       <x:c r="K51" s="35" t="str"/>
-      <x:c r="L51" s="36" t="str">
-        <x:v>Beginner CSF pathway landmark; activated for future manual annotation.</x:v>
-      </x:c>
+      <x:c r="L51" s="36" t="str"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="33" t="str">
@@ -2248,29 +2254,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C52" s="35" t="str">
-        <x:v>lateral_ventricle</x:v>
+        <x:v>interventricular_foramen_foramen_of_monro</x:v>
       </x:c>
       <x:c r="D52" s="35" t="str">
-        <x:v>Lateral Ventricle</x:v>
+        <x:v>Interventricular foramen (foramen of Monro)</x:v>
       </x:c>
       <x:c r="E52" s="35" t="str">
-        <x:v>csf_spaces; ventricles</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F52" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G52" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H52" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I52" s="35" t="str">
-        <x:v>annotations/001_lateral_ventricle.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G52" s="35" t="str"/>
+      <x:c r="H52" s="35" t="str"/>
+      <x:c r="I52" s="35" t="str"/>
       <x:c r="J52" s="35" t="str"/>
       <x:c r="K52" s="35" t="str"/>
-      <x:c r="L52" s="36" t="str"/>
+      <x:c r="L52" s="36" t="str">
+        <x:v>Beginner CSF pathway landmark; activated for future manual annotation.</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="33" t="str">
@@ -2280,25 +2282,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C53" s="35" t="str">
-        <x:v>lentiform_nucleus</x:v>
+        <x:v>lateral_ventricle</x:v>
       </x:c>
       <x:c r="D53" s="35" t="str">
-        <x:v>Lentiform nucleus</x:v>
+        <x:v>Lateral Ventricle</x:v>
       </x:c>
       <x:c r="E53" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>csf_spaces; ventricles</x:v>
       </x:c>
       <x:c r="F53" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G53" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H53" s="35" t="str">
-        <x:v>accepted</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I53" s="35" t="str">
-        <x:v>annotations/065_lentiform_nucleus.nii.gz</x:v>
+        <x:v>annotations/001_lateral_ventricle.nii.gz</x:v>
       </x:c>
       <x:c r="J53" s="35" t="str"/>
       <x:c r="K53" s="35" t="str"/>
@@ -2309,28 +2311,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B54" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C54" s="35" t="str">
-        <x:v>lingual_gyrus</x:v>
+        <x:v>lentiform_nucleus</x:v>
       </x:c>
       <x:c r="D54" s="35" t="str">
-        <x:v>Lingual gyrus</x:v>
+        <x:v>Lentiform nucleus</x:v>
       </x:c>
       <x:c r="E54" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="F54" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G54" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H54" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I54" s="35" t="str">
-        <x:v>annotations/016_lingual_gyrus.nii.gz</x:v>
+        <x:v>annotations/065_lentiform_nucleus.nii.gz</x:v>
       </x:c>
       <x:c r="J54" s="35" t="str"/>
       <x:c r="K54" s="35" t="str"/>
@@ -2341,23 +2343,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B55" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C55" s="35" t="str">
-        <x:v>mammillary_bodies</x:v>
+        <x:v>lingual_gyrus</x:v>
       </x:c>
       <x:c r="D55" s="35" t="str">
-        <x:v>Mammillary bodies</x:v>
+        <x:v>Lingual gyrus</x:v>
       </x:c>
       <x:c r="E55" s="35" t="str">
-        <x:v>limbic; midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F55" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G55" s="35" t="str"/>
-      <x:c r="H55" s="35" t="str"/>
-      <x:c r="I55" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G55" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H55" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I55" s="35" t="str">
+        <x:v>annotations/016_lingual_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J55" s="35" t="str"/>
       <x:c r="K55" s="35" t="str"/>
       <x:c r="L55" s="36" t="str"/>
@@ -2367,28 +2375,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B56" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C56" s="35" t="str">
-        <x:v>marginal_sulcus_pars_marginalis</x:v>
+        <x:v>mammillary_bodies</x:v>
       </x:c>
       <x:c r="D56" s="35" t="str">
-        <x:v>Marginal sulcus (pars marginalis)</x:v>
+        <x:v>Mammillary bodies</x:v>
       </x:c>
       <x:c r="E56" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>limbic; midline</x:v>
       </x:c>
       <x:c r="F56" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G56" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H56" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I56" s="35" t="str">
-        <x:v>annotations/083_marginal_sulcus_pars_marginalis.nii.gz</x:v>
+        <x:v>annotations/052_mammillary_bodies.nii.gz</x:v>
       </x:c>
       <x:c r="J56" s="35" t="str"/>
       <x:c r="K56" s="35" t="str"/>
@@ -2402,20 +2410,26 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C57" s="35" t="str">
-        <x:v>meckel_s_cave</x:v>
+        <x:v>marginal_sulcus_pars_marginalis</x:v>
       </x:c>
       <x:c r="D57" s="35" t="str">
-        <x:v>Meckel's cave</x:v>
+        <x:v>Marginal sulcus (pars marginalis)</x:v>
       </x:c>
       <x:c r="E57" s="35" t="str">
-        <x:v>skull_base; cranial_nerves; csf_spaces</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="F57" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G57" s="35" t="str"/>
-      <x:c r="H57" s="35" t="str"/>
-      <x:c r="I57" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G57" s="35" t="str">
+        <x:v>freesurfer_seed_split</x:v>
+      </x:c>
+      <x:c r="H57" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I57" s="35" t="str">
+        <x:v>annotations/083_marginal_sulcus_pars_marginalis.nii.gz</x:v>
+      </x:c>
       <x:c r="J57" s="35" t="str"/>
       <x:c r="K57" s="35" t="str"/>
       <x:c r="L57" s="36" t="str"/>
@@ -2425,16 +2439,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B58" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C58" s="35" t="str">
-        <x:v>median_interhemispheric_fissure</x:v>
+        <x:v>meckel_s_cave</x:v>
       </x:c>
       <x:c r="D58" s="35" t="str">
-        <x:v>Median interhemispheric fissure</x:v>
+        <x:v>Meckel's cave</x:v>
       </x:c>
       <x:c r="E58" s="35" t="str">
-        <x:v>csf_spaces; midline</x:v>
+        <x:v>skull_base; cranial_nerves; csf_spaces</x:v>
       </x:c>
       <x:c r="F58" s="35" t="str">
         <x:v>no</x:v>
@@ -2454,26 +2468,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C59" s="35" t="str">
-        <x:v>medulla_oblongata</x:v>
+        <x:v>median_interhemispheric_fissure</x:v>
       </x:c>
       <x:c r="D59" s="35" t="str">
-        <x:v>Medulla oblongata</x:v>
+        <x:v>Median interhemispheric fissure</x:v>
       </x:c>
       <x:c r="E59" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>csf_spaces; midline</x:v>
       </x:c>
       <x:c r="F59" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G59" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H59" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I59" s="35" t="str">
-        <x:v>annotations/029_medulla_oblongata.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G59" s="35" t="str"/>
+      <x:c r="H59" s="35" t="str"/>
+      <x:c r="I59" s="35" t="str"/>
       <x:c r="J59" s="35" t="str"/>
       <x:c r="K59" s="35" t="str"/>
       <x:c r="L59" s="36" t="str"/>
@@ -2486,10 +2494,10 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C60" s="35" t="str">
-        <x:v>midbrain</x:v>
+        <x:v>medulla_oblongata</x:v>
       </x:c>
       <x:c r="D60" s="35" t="str">
-        <x:v>Midbrain</x:v>
+        <x:v>Medulla oblongata</x:v>
       </x:c>
       <x:c r="E60" s="35" t="str">
         <x:v>brainstem</x:v>
@@ -2504,7 +2512,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I60" s="35" t="str">
-        <x:v>annotations/054_midbrain.nii.gz</x:v>
+        <x:v>annotations/029_medulla_oblongata.nii.gz</x:v>
       </x:c>
       <x:c r="J60" s="35" t="str"/>
       <x:c r="K60" s="35" t="str"/>
@@ -2518,39 +2526,45 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C61" s="35" t="str">
-        <x:v>middle_cerebellar_peduncle</x:v>
+        <x:v>midbrain</x:v>
       </x:c>
       <x:c r="D61" s="35" t="str">
-        <x:v>Middle cerebellar peduncle</x:v>
+        <x:v>Midbrain</x:v>
       </x:c>
       <x:c r="E61" s="35" t="str">
-        <x:v>white_matter; cerebellum; brainstem</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="F61" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G61" s="35" t="str"/>
-      <x:c r="H61" s="35" t="str"/>
-      <x:c r="I61" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G61" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H61" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I61" s="35" t="str">
+        <x:v>annotations/054_midbrain.nii.gz</x:v>
+      </x:c>
       <x:c r="J61" s="35" t="str"/>
       <x:c r="K61" s="35" t="str"/>
       <x:c r="L61" s="36" t="str"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B62" s="34" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C62" s="35" t="str">
-        <x:v>middle_temporal_gyrus</x:v>
+        <x:v>middle_cerebellar_peduncle</x:v>
       </x:c>
       <x:c r="D62" s="35" t="str">
-        <x:v>Middle temporal gyrus</x:v>
+        <x:v>Middle cerebellar peduncle</x:v>
       </x:c>
       <x:c r="E62" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>white_matter; cerebellum; brainstem</x:v>
       </x:c>
       <x:c r="F62" s="35" t="str">
         <x:v>no</x:v>
@@ -2564,19 +2578,19 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B63" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C63" s="35" t="str">
-        <x:v>nodule_of_the_cerebellum</x:v>
+        <x:v>middle_temporal_gyrus</x:v>
       </x:c>
       <x:c r="D63" s="35" t="str">
-        <x:v>Nodule of the cerebellum</x:v>
+        <x:v>Middle temporal gyrus</x:v>
       </x:c>
       <x:c r="E63" s="35" t="str">
-        <x:v>cerebellum; midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F63" s="35" t="str">
         <x:v>no</x:v>
@@ -2596,26 +2610,20 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C64" s="35" t="str">
-        <x:v>nucleus_accumbens</x:v>
+        <x:v>nodule_of_the_cerebellum</x:v>
       </x:c>
       <x:c r="D64" s="35" t="str">
-        <x:v>Nucleus accumbens</x:v>
+        <x:v>Nodule of the cerebellum</x:v>
       </x:c>
       <x:c r="E64" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>cerebellum; midline</x:v>
       </x:c>
       <x:c r="F64" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G64" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H64" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I64" s="35" t="str">
-        <x:v>annotations/010_nucleus_accumbens.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G64" s="35" t="str"/>
+      <x:c r="H64" s="35" t="str"/>
+      <x:c r="I64" s="35" t="str"/>
       <x:c r="J64" s="35" t="str"/>
       <x:c r="K64" s="35" t="str"/>
       <x:c r="L64" s="36" t="str"/>
@@ -2625,28 +2633,28 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B65" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C65" s="35" t="str">
-        <x:v>occipital_horn_of_the_lateral_ventricle</x:v>
+        <x:v>nucleus_accumbens</x:v>
       </x:c>
       <x:c r="D65" s="35" t="str">
-        <x:v>Occipital horn of the lateral ventricle</x:v>
+        <x:v>Nucleus accumbens</x:v>
       </x:c>
       <x:c r="E65" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="F65" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G65" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H65" s="35" t="str">
-        <x:v>accepted</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I65" s="35" t="str">
-        <x:v>annotations/076_occipital_horn_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/010_nucleus_accumbens.nii.gz</x:v>
       </x:c>
       <x:c r="J65" s="35" t="str"/>
       <x:c r="K65" s="35" t="str"/>
@@ -2660,13 +2668,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C66" s="35" t="str">
-        <x:v>occipital_lobe</x:v>
+        <x:v>occipital_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D66" s="35" t="str">
-        <x:v>Occipital lobe</x:v>
+        <x:v>Occipital horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E66" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F66" s="35" t="str">
         <x:v>yes</x:v>
@@ -2678,7 +2686,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I66" s="35" t="str">
-        <x:v>annotations/074_occipital_lobe.nii.gz</x:v>
+        <x:v>annotations/076_occipital_horn_of_the_lateral_ventricle.nii.gz</x:v>
       </x:c>
       <x:c r="J66" s="35" t="str"/>
       <x:c r="K66" s="35" t="str"/>
@@ -2692,25 +2700,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C67" s="35" t="str">
-        <x:v>optic_chiasm</x:v>
+        <x:v>occipital_lobe</x:v>
       </x:c>
       <x:c r="D67" s="35" t="str">
-        <x:v>Optic chiasm</x:v>
+        <x:v>Occipital lobe</x:v>
       </x:c>
       <x:c r="E67" s="35" t="str">
-        <x:v>cranial_nerves; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F67" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G67" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H67" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I67" s="35" t="str">
-        <x:v>annotations/012_optic_chiasm.nii.gz</x:v>
+        <x:v>annotations/074_occipital_lobe.nii.gz</x:v>
       </x:c>
       <x:c r="J67" s="35" t="str"/>
       <x:c r="K67" s="35" t="str"/>
@@ -2724,57 +2732,57 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C68" s="35" t="str">
-        <x:v>optic_nerve</x:v>
+        <x:v>optic_chiasm</x:v>
       </x:c>
       <x:c r="D68" s="35" t="str">
-        <x:v>Optic nerve</x:v>
+        <x:v>Optic chiasm</x:v>
       </x:c>
       <x:c r="E68" s="35" t="str">
-        <x:v>cranial_nerves; skull_base; orbit</x:v>
+        <x:v>cranial_nerves; skull_base</x:v>
       </x:c>
       <x:c r="F68" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G68" s="35" t="str"/>
-      <x:c r="H68" s="35" t="str"/>
-      <x:c r="I68" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G68" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H68" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I68" s="35" t="str">
+        <x:v>annotations/012_optic_chiasm.nii.gz</x:v>
+      </x:c>
       <x:c r="J68" s="35" t="str"/>
       <x:c r="K68" s="35" t="str"/>
-      <x:c r="L68" s="36" t="str">
-        <x:v>High-yield anterior skull base/orbital apex structure adjacent to the optic chiasm.</x:v>
-      </x:c>
+      <x:c r="L68" s="36" t="str"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B69" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C69" s="35" t="str">
-        <x:v>orbitofrontal_cortex</x:v>
+        <x:v>optic_nerve</x:v>
       </x:c>
       <x:c r="D69" s="35" t="str">
-        <x:v>Orbitofrontal cortex</x:v>
+        <x:v>Optic nerve</x:v>
       </x:c>
       <x:c r="E69" s="35" t="str">
-        <x:v>cortex; skull_base</x:v>
+        <x:v>cranial_nerves; skull_base; orbit</x:v>
       </x:c>
       <x:c r="F69" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G69" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H69" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I69" s="35" t="str">
-        <x:v>annotations/090_orbitofrontal_cortex.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G69" s="35" t="str"/>
+      <x:c r="H69" s="35" t="str"/>
+      <x:c r="I69" s="35" t="str"/>
       <x:c r="J69" s="35" t="str"/>
       <x:c r="K69" s="35" t="str"/>
-      <x:c r="L69" s="36" t="str"/>
+      <x:c r="L69" s="36" t="str">
+        <x:v>High-yield anterior skull base/orbital apex structure adjacent to the optic chiasm.</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="33" t="str">
@@ -2784,13 +2792,13 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C70" s="35" t="str">
-        <x:v>parahippocampal_gyrus</x:v>
+        <x:v>orbitofrontal_cortex</x:v>
       </x:c>
       <x:c r="D70" s="35" t="str">
-        <x:v>Parahippocampal gyrus</x:v>
+        <x:v>Orbitofrontal cortex</x:v>
       </x:c>
       <x:c r="E70" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex; skull_base</x:v>
       </x:c>
       <x:c r="F70" s="35" t="str">
         <x:v>yes</x:v>
@@ -2802,7 +2810,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I70" s="35" t="str">
-        <x:v>annotations/089_parahippocampal_gyrus.nii.gz</x:v>
+        <x:v>annotations/090_orbitofrontal_cortex.nii.gz</x:v>
       </x:c>
       <x:c r="J70" s="35" t="str"/>
       <x:c r="K70" s="35" t="str"/>
@@ -2813,60 +2821,60 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B71" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C71" s="35" t="str">
-        <x:v>parietal_lobe</x:v>
+        <x:v>parahippocampal_gyrus</x:v>
       </x:c>
       <x:c r="D71" s="35" t="str">
-        <x:v>Parietal lobe</x:v>
+        <x:v>Parahippocampal gyrus</x:v>
       </x:c>
       <x:c r="E71" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="F71" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G71" s="35" t="str"/>
-      <x:c r="H71" s="35" t="str"/>
-      <x:c r="I71" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G71" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H71" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I71" s="35" t="str">
+        <x:v>annotations/089_parahippocampal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J71" s="35" t="str"/>
       <x:c r="K71" s="35" t="str"/>
-      <x:c r="L71" s="36" t="str">
-        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
-      </x:c>
+      <x:c r="L71" s="36" t="str"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B72" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C72" s="35" t="str">
-        <x:v>parieto_occipital_sulcus</x:v>
+        <x:v>parietal_lobe</x:v>
       </x:c>
       <x:c r="D72" s="35" t="str">
-        <x:v>Parieto-occipital sulcus</x:v>
+        <x:v>Parietal lobe</x:v>
       </x:c>
       <x:c r="E72" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="F72" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G72" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H72" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I72" s="35" t="str">
-        <x:v>annotations/092_parieto_occipital_sulcus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G72" s="35" t="str"/>
+      <x:c r="H72" s="35" t="str"/>
+      <x:c r="I72" s="35" t="str"/>
       <x:c r="J72" s="35" t="str"/>
       <x:c r="K72" s="35" t="str"/>
-      <x:c r="L72" s="36" t="str"/>
+      <x:c r="L72" s="36" t="str">
+        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
+      </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="33" t="str">
@@ -2876,10 +2884,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C73" s="35" t="str">
-        <x:v>pars_opercularis</x:v>
+        <x:v>parieto_occipital_sulcus</x:v>
       </x:c>
       <x:c r="D73" s="35" t="str">
-        <x:v>Pars opercularis</x:v>
+        <x:v>Parieto-occipital sulcus</x:v>
       </x:c>
       <x:c r="E73" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2888,13 +2896,13 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G73" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H73" s="35" t="str">
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I73" s="35" t="str">
-        <x:v>annotations/017_pars_opercularis.nii.gz</x:v>
+        <x:v>annotations/092_parieto_occipital_sulcus.nii.gz</x:v>
       </x:c>
       <x:c r="J73" s="35" t="str"/>
       <x:c r="K73" s="35" t="str"/>
@@ -2908,10 +2916,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C74" s="35" t="str">
-        <x:v>pars_orbitalis</x:v>
+        <x:v>pars_opercularis</x:v>
       </x:c>
       <x:c r="D74" s="35" t="str">
-        <x:v>Pars orbitalis</x:v>
+        <x:v>Pars opercularis</x:v>
       </x:c>
       <x:c r="E74" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2926,7 +2934,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I74" s="35" t="str">
-        <x:v>annotations/018_pars_orbitalis.nii.gz</x:v>
+        <x:v>annotations/017_pars_opercularis.nii.gz</x:v>
       </x:c>
       <x:c r="J74" s="35" t="str"/>
       <x:c r="K74" s="35" t="str"/>
@@ -2940,10 +2948,10 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C75" s="35" t="str">
-        <x:v>pars_triangularis</x:v>
+        <x:v>pars_orbitalis</x:v>
       </x:c>
       <x:c r="D75" s="35" t="str">
-        <x:v>Pars triangularis</x:v>
+        <x:v>Pars orbitalis</x:v>
       </x:c>
       <x:c r="E75" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2958,7 +2966,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I75" s="35" t="str">
-        <x:v>annotations/019_pars_triangularis.nii.gz</x:v>
+        <x:v>annotations/018_pars_orbitalis.nii.gz</x:v>
       </x:c>
       <x:c r="J75" s="35" t="str"/>
       <x:c r="K75" s="35" t="str"/>
@@ -2969,23 +2977,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B76" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C76" s="35" t="str">
-        <x:v>pineal_gland</x:v>
+        <x:v>pars_triangularis</x:v>
       </x:c>
       <x:c r="D76" s="35" t="str">
-        <x:v>Pineal gland</x:v>
+        <x:v>Pars triangularis</x:v>
       </x:c>
       <x:c r="E76" s="35" t="str">
-        <x:v>midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F76" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G76" s="35" t="str"/>
-      <x:c r="H76" s="35" t="str"/>
-      <x:c r="I76" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G76" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H76" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I76" s="35" t="str">
+        <x:v>annotations/019_pars_triangularis.nii.gz</x:v>
+      </x:c>
       <x:c r="J76" s="35" t="str"/>
       <x:c r="K76" s="35" t="str"/>
       <x:c r="L76" s="36" t="str"/>
@@ -2998,13 +3012,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C77" s="35" t="str">
-        <x:v>pituitary_fossa</x:v>
+        <x:v>pineal_gland</x:v>
       </x:c>
       <x:c r="D77" s="35" t="str">
-        <x:v>Pituitary fossa</x:v>
+        <x:v>Pineal gland</x:v>
       </x:c>
       <x:c r="E77" s="35" t="str">
-        <x:v>skull_base; midline</x:v>
+        <x:v>midline</x:v>
       </x:c>
       <x:c r="F77" s="35" t="str">
         <x:v>no</x:v>
@@ -3024,26 +3038,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C78" s="35" t="str">
-        <x:v>pons</x:v>
+        <x:v>pituitary_fossa</x:v>
       </x:c>
       <x:c r="D78" s="35" t="str">
-        <x:v>Pons</x:v>
+        <x:v>Pituitary fossa</x:v>
       </x:c>
       <x:c r="E78" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>skull_base; midline</x:v>
       </x:c>
       <x:c r="F78" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G78" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H78" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I78" s="35" t="str">
-        <x:v>annotations/040_pons.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G78" s="35" t="str"/>
+      <x:c r="H78" s="35" t="str"/>
+      <x:c r="I78" s="35" t="str"/>
       <x:c r="J78" s="35" t="str"/>
       <x:c r="K78" s="35" t="str"/>
       <x:c r="L78" s="36" t="str"/>
@@ -3056,25 +3064,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C79" s="35" t="str">
-        <x:v>postcentral_gyrus</x:v>
+        <x:v>pons</x:v>
       </x:c>
       <x:c r="D79" s="35" t="str">
-        <x:v>Postcentral gyrus</x:v>
+        <x:v>Pons</x:v>
       </x:c>
       <x:c r="E79" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="F79" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G79" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
+        <x:v>accepted_annotation</x:v>
       </x:c>
       <x:c r="H79" s="35" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>accepted</x:v>
       </x:c>
       <x:c r="I79" s="35" t="str">
-        <x:v>annotations/020_postcentral_gyrus.nii.gz</x:v>
+        <x:v>annotations/040_pons.nii.gz</x:v>
       </x:c>
       <x:c r="J79" s="35" t="str"/>
       <x:c r="K79" s="35" t="str"/>
@@ -3085,16 +3093,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B80" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C80" s="35" t="str">
-        <x:v>posterior_cingulate_gyrus</x:v>
+        <x:v>postcentral_gyrus</x:v>
       </x:c>
       <x:c r="D80" s="35" t="str">
-        <x:v>Posterior cingulate gyrus</x:v>
+        <x:v>Postcentral gyrus</x:v>
       </x:c>
       <x:c r="E80" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F80" s="35" t="str">
         <x:v>yes</x:v>
@@ -3106,7 +3114,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I80" s="35" t="str">
-        <x:v>annotations/021_posterior_cingulate_gyrus.nii.gz</x:v>
+        <x:v>annotations/020_postcentral_gyrus.nii.gz</x:v>
       </x:c>
       <x:c r="J80" s="35" t="str"/>
       <x:c r="K80" s="35" t="str"/>
@@ -3120,20 +3128,26 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C81" s="35" t="str">
-        <x:v>posterior_commissure</x:v>
+        <x:v>posterior_cingulate_gyrus</x:v>
       </x:c>
       <x:c r="D81" s="35" t="str">
-        <x:v>Posterior commissure</x:v>
+        <x:v>Posterior cingulate gyrus</x:v>
       </x:c>
       <x:c r="E81" s="35" t="str">
-        <x:v>white_matter; midline; brainstem</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="F81" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G81" s="35" t="str"/>
-      <x:c r="H81" s="35" t="str"/>
-      <x:c r="I81" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G81" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H81" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I81" s="35" t="str">
+        <x:v>annotations/021_posterior_cingulate_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J81" s="35" t="str"/>
       <x:c r="K81" s="35" t="str"/>
       <x:c r="L81" s="36" t="str"/>
@@ -3143,16 +3157,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B82" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C82" s="35" t="str">
-        <x:v>posterior_limb_of_the_internal_capsule</x:v>
+        <x:v>posterior_commissure</x:v>
       </x:c>
       <x:c r="D82" s="35" t="str">
-        <x:v>Posterior limb of the internal capsule</x:v>
+        <x:v>Posterior commissure</x:v>
       </x:c>
       <x:c r="E82" s="35" t="str">
-        <x:v>white_matter; basal_ganglia</x:v>
+        <x:v>white_matter; midline; brainstem</x:v>
       </x:c>
       <x:c r="F82" s="35" t="str">
         <x:v>no</x:v>
@@ -3172,26 +3186,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C83" s="35" t="str">
-        <x:v>precentral_gyrus</x:v>
+        <x:v>posterior_limb_of_the_internal_capsule</x:v>
       </x:c>
       <x:c r="D83" s="35" t="str">
-        <x:v>Precentral gyrus</x:v>
+        <x:v>Posterior limb of the internal capsule</x:v>
       </x:c>
       <x:c r="E83" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>white_matter; basal_ganglia</x:v>
       </x:c>
       <x:c r="F83" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G83" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H83" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I83" s="35" t="str">
-        <x:v>annotations/022_precentral_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G83" s="35" t="str"/>
+      <x:c r="H83" s="35" t="str"/>
+      <x:c r="I83" s="35" t="str"/>
       <x:c r="J83" s="35" t="str"/>
       <x:c r="K83" s="35" t="str"/>
       <x:c r="L83" s="36" t="str"/>
@@ -3201,13 +3209,13 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B84" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C84" s="35" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>precentral_gyrus</x:v>
       </x:c>
       <x:c r="D84" s="35" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>Precentral gyrus</x:v>
       </x:c>
       <x:c r="E84" s="35" t="str">
         <x:v>cortex</x:v>
@@ -3222,7 +3230,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I84" s="35" t="str">
-        <x:v>annotations/023_precuneus.nii.gz</x:v>
+        <x:v>annotations/022_precentral_gyrus.nii.gz</x:v>
       </x:c>
       <x:c r="J84" s="35" t="str"/>
       <x:c r="K84" s="35" t="str"/>
@@ -3233,23 +3241,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B85" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C85" s="35" t="str">
-        <x:v>premedullary_cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="D85" s="35" t="str">
-        <x:v>Premedullary cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="E85" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F85" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G85" s="35" t="str"/>
-      <x:c r="H85" s="35" t="str"/>
-      <x:c r="I85" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G85" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H85" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I85" s="35" t="str">
+        <x:v>annotations/023_precuneus.nii.gz</x:v>
+      </x:c>
       <x:c r="J85" s="35" t="str"/>
       <x:c r="K85" s="35" t="str"/>
       <x:c r="L85" s="36" t="str"/>
@@ -3262,10 +3276,10 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C86" s="35" t="str">
-        <x:v>prepontine_cistern</x:v>
+        <x:v>premedullary_cistern</x:v>
       </x:c>
       <x:c r="D86" s="35" t="str">
-        <x:v>Prepontine cistern</x:v>
+        <x:v>Premedullary cistern</x:v>
       </x:c>
       <x:c r="E86" s="35" t="str">
         <x:v>csf_spaces; brainstem</x:v>
@@ -3288,26 +3302,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C87" s="35" t="str">
-        <x:v>putamen</x:v>
+        <x:v>prepontine_cistern</x:v>
       </x:c>
       <x:c r="D87" s="35" t="str">
-        <x:v>Putamen</x:v>
+        <x:v>Prepontine cistern</x:v>
       </x:c>
       <x:c r="E87" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F87" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G87" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H87" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I87" s="35" t="str">
-        <x:v>annotations/004_putamen.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G87" s="35" t="str"/>
+      <x:c r="H87" s="35" t="str"/>
+      <x:c r="I87" s="35" t="str"/>
       <x:c r="J87" s="35" t="str"/>
       <x:c r="K87" s="35" t="str"/>
       <x:c r="L87" s="36" t="str"/>
@@ -3320,20 +3328,26 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C88" s="35" t="str">
-        <x:v>quadrigeminal_cistern</x:v>
+        <x:v>putamen</x:v>
       </x:c>
       <x:c r="D88" s="35" t="str">
-        <x:v>Quadrigeminal cistern</x:v>
+        <x:v>Putamen</x:v>
       </x:c>
       <x:c r="E88" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="F88" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G88" s="35" t="str"/>
-      <x:c r="H88" s="35" t="str"/>
-      <x:c r="I88" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G88" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H88" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I88" s="35" t="str">
+        <x:v>annotations/004_putamen.nii.gz</x:v>
+      </x:c>
       <x:c r="J88" s="35" t="str"/>
       <x:c r="K88" s="35" t="str"/>
       <x:c r="L88" s="36" t="str"/>
@@ -3343,16 +3357,16 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B89" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
-        <x:v>rostrum_of_the_corpus_callosum</x:v>
+        <x:v>quadrigeminal_cistern</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>Rostrum of the corpus callosum</x:v>
+        <x:v>Quadrigeminal cistern</x:v>
       </x:c>
       <x:c r="E89" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="F89" s="35" t="str">
         <x:v>no</x:v>
@@ -3362,9 +3376,7 @@
       <x:c r="I89" s="35" t="str"/>
       <x:c r="J89" s="35" t="str"/>
       <x:c r="K89" s="35" t="str"/>
-      <x:c r="L89" s="36" t="str">
-        <x:v>Added from browser-created accepted mask; review in viewer/ITK-SNAP.</x:v>
-      </x:c>
+      <x:c r="L89" s="36" t="str"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="33" t="str">
@@ -3374,13 +3386,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
-        <x:v>septum_pellucidum</x:v>
+        <x:v>rostrum_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>Septum pellucidum</x:v>
+        <x:v>Rostrum of the corpus callosum</x:v>
       </x:c>
       <x:c r="E90" s="35" t="str">
-        <x:v>midline; ventricles; csf_spaces</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F90" s="35" t="str">
         <x:v>yes</x:v>
@@ -3392,11 +3404,13 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I90" s="35" t="str">
-        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
+        <x:v>annotations/106_rostrum_of_the_corpus_callosum.nii.gz</x:v>
       </x:c>
       <x:c r="J90" s="35" t="str"/>
       <x:c r="K90" s="35" t="str"/>
-      <x:c r="L90" s="36" t="str"/>
+      <x:c r="L90" s="36" t="str">
+        <x:v>Added from browser-created accepted mask; review in viewer/ITK-SNAP.</x:v>
+      </x:c>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="33" t="str">
@@ -3406,13 +3420,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
-        <x:v>splenium_of_the_corpus_callosum</x:v>
+        <x:v>septum_pellucidum</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>Splenium of the corpus callosum</x:v>
+        <x:v>Septum pellucidum</x:v>
       </x:c>
       <x:c r="E91" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F91" s="35" t="str">
         <x:v>yes</x:v>
@@ -3424,7 +3438,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I91" s="35" t="str">
-        <x:v>annotations/075_splenium_of_the_corpus_callosum.nii.gz</x:v>
+        <x:v>annotations/071_septum_pellucidum.nii.gz</x:v>
       </x:c>
       <x:c r="J91" s="35" t="str"/>
       <x:c r="K91" s="35" t="str"/>
@@ -3438,57 +3452,57 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
-        <x:v>subthalamic_region</x:v>
+        <x:v>splenium_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>Subthalamic region</x:v>
+        <x:v>Splenium of the corpus callosum</x:v>
       </x:c>
       <x:c r="E92" s="35" t="str">
-        <x:v>deep_gray; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="F92" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G92" s="35" t="str"/>
-      <x:c r="H92" s="35" t="str"/>
-      <x:c r="I92" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G92" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H92" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I92" s="35" t="str">
+        <x:v>annotations/075_splenium_of_the_corpus_callosum.nii.gz</x:v>
+      </x:c>
       <x:c r="J92" s="35" t="str"/>
       <x:c r="K92" s="35" t="str"/>
-      <x:c r="L92" s="36" t="str">
-        <x:v>Optional beginner-to-intermediate deep gray landmark if it can be shown cleanly on this T1.</x:v>
-      </x:c>
+      <x:c r="L92" s="36" t="str"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B93" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
-        <x:v>superior_frontal_gyrus</x:v>
+        <x:v>subthalamic_region</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>Superior frontal gyrus</x:v>
+        <x:v>Subthalamic region</x:v>
       </x:c>
       <x:c r="E93" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>deep_gray; basal_ganglia</x:v>
       </x:c>
       <x:c r="F93" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G93" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H93" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I93" s="35" t="str">
-        <x:v>annotations/024_superior_frontal_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G93" s="35" t="str"/>
+      <x:c r="H93" s="35" t="str"/>
+      <x:c r="I93" s="35" t="str"/>
       <x:c r="J93" s="35" t="str"/>
       <x:c r="K93" s="35" t="str"/>
-      <x:c r="L93" s="36" t="str"/>
+      <x:c r="L93" s="36" t="str">
+        <x:v>Optional beginner-to-intermediate deep gray landmark if it can be shown cleanly on this T1.</x:v>
+      </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="33" t="str">
@@ -3498,39 +3512,45 @@
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
-        <x:v>superior_orbital_fissure</x:v>
+        <x:v>superior_frontal_gyrus</x:v>
       </x:c>
       <x:c r="D94" s="35" t="str">
-        <x:v>Superior orbital fissure</x:v>
+        <x:v>Superior frontal gyrus</x:v>
       </x:c>
       <x:c r="E94" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F94" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G94" s="35" t="str"/>
-      <x:c r="H94" s="35" t="str"/>
-      <x:c r="I94" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G94" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H94" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I94" s="35" t="str">
+        <x:v>annotations/024_superior_frontal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J94" s="35" t="str"/>
       <x:c r="K94" s="35" t="str"/>
       <x:c r="L94" s="36" t="str"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="33" t="str">
-        <x:v>no</x:v>
+        <x:v>yes</x:v>
       </x:c>
       <x:c r="B95" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C95" s="35" t="str">
-        <x:v>superior_temporal_gyrus</x:v>
+        <x:v>superior_orbital_fissure</x:v>
       </x:c>
       <x:c r="D95" s="35" t="str">
-        <x:v>Superior temporal gyrus</x:v>
+        <x:v>Superior orbital fissure</x:v>
       </x:c>
       <x:c r="E95" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="F95" s="35" t="str">
         <x:v>no</x:v>
@@ -3544,32 +3564,26 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="33" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="B96" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C96" s="35" t="str">
-        <x:v>supramarginal_gyrus</x:v>
+        <x:v>superior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="D96" s="35" t="str">
-        <x:v>Supramarginal gyrus</x:v>
+        <x:v>Superior temporal gyrus</x:v>
       </x:c>
       <x:c r="E96" s="35" t="str">
         <x:v>cortex</x:v>
       </x:c>
       <x:c r="F96" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G96" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H96" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I96" s="35" t="str">
-        <x:v>annotations/025_supramarginal_gyrus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G96" s="35" t="str"/>
+      <x:c r="H96" s="35" t="str"/>
+      <x:c r="I96" s="35" t="str"/>
       <x:c r="J96" s="35" t="str"/>
       <x:c r="K96" s="35" t="str"/>
       <x:c r="L96" s="36" t="str"/>
@@ -3579,23 +3593,29 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B97" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C97" s="35" t="str">
-        <x:v>suprasellar_cistern</x:v>
+        <x:v>supramarginal_gyrus</x:v>
       </x:c>
       <x:c r="D97" s="35" t="str">
-        <x:v>Suprasellar cistern</x:v>
+        <x:v>Supramarginal gyrus</x:v>
       </x:c>
       <x:c r="E97" s="35" t="str">
-        <x:v>csf_spaces; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F97" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G97" s="35" t="str"/>
-      <x:c r="H97" s="35" t="str"/>
-      <x:c r="I97" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G97" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H97" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I97" s="35" t="str">
+        <x:v>annotations/025_supramarginal_gyrus.nii.gz</x:v>
+      </x:c>
       <x:c r="J97" s="35" t="str"/>
       <x:c r="K97" s="35" t="str"/>
       <x:c r="L97" s="36" t="str"/>
@@ -3608,26 +3628,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C98" s="35" t="str">
-        <x:v>sylvian_fissure</x:v>
+        <x:v>suprasellar_cistern</x:v>
       </x:c>
       <x:c r="D98" s="35" t="str">
-        <x:v>Sylvian fissure</x:v>
+        <x:v>Suprasellar cistern</x:v>
       </x:c>
       <x:c r="E98" s="35" t="str">
-        <x:v>csf_spaces; cortex</x:v>
+        <x:v>csf_spaces; skull_base</x:v>
       </x:c>
       <x:c r="F98" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G98" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
-      </x:c>
-      <x:c r="H98" s="35" t="str">
-        <x:v>accepted</x:v>
-      </x:c>
-      <x:c r="I98" s="35" t="str">
-        <x:v>annotations/051_sylvian_fissure.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G98" s="35" t="str"/>
+      <x:c r="H98" s="35" t="str"/>
+      <x:c r="I98" s="35" t="str"/>
       <x:c r="J98" s="35" t="str"/>
       <x:c r="K98" s="35" t="str"/>
       <x:c r="L98" s="36" t="str"/>
@@ -3640,13 +3654,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C99" s="35" t="str">
-        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>sylvian_fissure</x:v>
       </x:c>
       <x:c r="D99" s="35" t="str">
-        <x:v>Temporal horn of the lateral ventricle</x:v>
+        <x:v>Sylvian fissure</x:v>
       </x:c>
       <x:c r="E99" s="35" t="str">
-        <x:v>ventricles; csf_spaces; deep_gray</x:v>
+        <x:v>csf_spaces; cortex</x:v>
       </x:c>
       <x:c r="F99" s="35" t="str">
         <x:v>yes</x:v>
@@ -3658,7 +3672,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I99" s="35" t="str">
-        <x:v>annotations/045_temporal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/051_sylvian_fissure.nii.gz</x:v>
       </x:c>
       <x:c r="J99" s="35" t="str"/>
       <x:c r="K99" s="35" t="str"/>
@@ -3672,80 +3686,86 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C100" s="35" t="str">
-        <x:v>temporal_lobe</x:v>
+        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D100" s="35" t="str">
-        <x:v>Temporal lobe</x:v>
+        <x:v>Temporal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E100" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces; deep_gray</x:v>
       </x:c>
       <x:c r="F100" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G100" s="35" t="str"/>
-      <x:c r="H100" s="35" t="str"/>
-      <x:c r="I100" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G100" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H100" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I100" s="35" t="str">
+        <x:v>annotations/045_temporal_horn_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J100" s="35" t="str"/>
       <x:c r="K100" s="35" t="str"/>
-      <x:c r="L100" s="36" t="str">
-        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
-      </x:c>
+      <x:c r="L100" s="36" t="str"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B101" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C101" s="35" t="str">
-        <x:v>temporal_pole</x:v>
+        <x:v>temporal_lobe</x:v>
       </x:c>
       <x:c r="D101" s="35" t="str">
-        <x:v>Temporal pole</x:v>
+        <x:v>Temporal lobe</x:v>
       </x:c>
       <x:c r="E101" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="F101" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G101" s="35" t="str">
-        <x:v>full_gyrus_composite</x:v>
-      </x:c>
-      <x:c r="H101" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I101" s="35" t="str">
-        <x:v>annotations/026_temporal_pole.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G101" s="35" t="str"/>
+      <x:c r="H101" s="35" t="str"/>
+      <x:c r="I101" s="35" t="str"/>
       <x:c r="J101" s="35" t="str"/>
       <x:c r="K101" s="35" t="str"/>
-      <x:c r="L101" s="36" t="str"/>
+      <x:c r="L101" s="36" t="str">
+        <x:v>Broad beginner lobar anatomy target; manually annotate once a mask is created.</x:v>
+      </x:c>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="33" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B102" s="34" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="C102" s="35" t="str">
-        <x:v>tentorium_cerebelli</x:v>
+        <x:v>temporal_pole</x:v>
       </x:c>
       <x:c r="D102" s="35" t="str">
-        <x:v>Tentorium cerebelli</x:v>
+        <x:v>Temporal pole</x:v>
       </x:c>
       <x:c r="E102" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="F102" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G102" s="35" t="str"/>
-      <x:c r="H102" s="35" t="str"/>
-      <x:c r="I102" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G102" s="35" t="str">
+        <x:v>full_gyrus_composite</x:v>
+      </x:c>
+      <x:c r="H102" s="35" t="str">
+        <x:v>needs_review</x:v>
+      </x:c>
+      <x:c r="I102" s="35" t="str">
+        <x:v>annotations/026_temporal_pole.nii.gz</x:v>
+      </x:c>
       <x:c r="J102" s="35" t="str"/>
       <x:c r="K102" s="35" t="str"/>
       <x:c r="L102" s="36" t="str"/>
@@ -3758,26 +3778,20 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C103" s="35" t="str">
-        <x:v>thalamus</x:v>
+        <x:v>tentorium_cerebelli</x:v>
       </x:c>
       <x:c r="D103" s="35" t="str">
-        <x:v>Thalamus</x:v>
+        <x:v>Tentorium cerebelli</x:v>
       </x:c>
       <x:c r="E103" s="35" t="str">
-        <x:v>deep_gray</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="F103" s="35" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="G103" s="35" t="str">
-        <x:v>freesurfer_seed_split</x:v>
-      </x:c>
-      <x:c r="H103" s="35" t="str">
-        <x:v>needs_review</x:v>
-      </x:c>
-      <x:c r="I103" s="35" t="str">
-        <x:v>annotations/002_thalamus.nii.gz</x:v>
-      </x:c>
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G103" s="35" t="str"/>
+      <x:c r="H103" s="35" t="str"/>
+      <x:c r="I103" s="35" t="str"/>
       <x:c r="J103" s="35" t="str"/>
       <x:c r="K103" s="35" t="str"/>
       <x:c r="L103" s="36" t="str"/>
@@ -3790,13 +3804,13 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C104" s="35" t="str">
-        <x:v>third_ventricle</x:v>
+        <x:v>thalamus</x:v>
       </x:c>
       <x:c r="D104" s="35" t="str">
-        <x:v>Third ventricle</x:v>
+        <x:v>Thalamus</x:v>
       </x:c>
       <x:c r="E104" s="35" t="str">
-        <x:v>ventricles; csf_spaces; midline</x:v>
+        <x:v>deep_gray</x:v>
       </x:c>
       <x:c r="F104" s="35" t="str">
         <x:v>yes</x:v>
@@ -3808,7 +3822,7 @@
         <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I104" s="35" t="str">
-        <x:v>annotations/006_third_ventricle.nii.gz</x:v>
+        <x:v>annotations/002_thalamus.nii.gz</x:v>
       </x:c>
       <x:c r="J104" s="35" t="str"/>
       <x:c r="K104" s="35" t="str"/>
@@ -3822,25 +3836,25 @@
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="C105" s="35" t="str">
-        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
+        <x:v>third_ventricle</x:v>
       </x:c>
       <x:c r="D105" s="35" t="str">
-        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
+        <x:v>Third ventricle</x:v>
       </x:c>
       <x:c r="E105" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; midline</x:v>
       </x:c>
       <x:c r="F105" s="35" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="G105" s="35" t="str">
-        <x:v>accepted_annotation</x:v>
+        <x:v>freesurfer_seed_split</x:v>
       </x:c>
       <x:c r="H105" s="35" t="str">
-        <x:v>accepted</x:v>
+        <x:v>needs_review</x:v>
       </x:c>
       <x:c r="I105" s="35" t="str">
-        <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
+        <x:v>annotations/006_third_ventricle.nii.gz</x:v>
       </x:c>
       <x:c r="J105" s="35" t="str"/>
       <x:c r="K105" s="35" t="str"/>
@@ -3851,65 +3865,97 @@
         <x:v>yes</x:v>
       </x:c>
       <x:c r="B106" s="34" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="C106" s="35" t="str">
-        <x:v>uncus</x:v>
+        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="D106" s="35" t="str">
-        <x:v>Uncus</x:v>
+        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
       </x:c>
       <x:c r="E106" s="35" t="str">
-        <x:v>limbic; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="F106" s="35" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="G106" s="35" t="str"/>
-      <x:c r="H106" s="35" t="str"/>
-      <x:c r="I106" s="35" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="G106" s="35" t="str">
+        <x:v>accepted_annotation</x:v>
+      </x:c>
+      <x:c r="H106" s="35" t="str">
+        <x:v>accepted</x:v>
+      </x:c>
+      <x:c r="I106" s="35" t="str">
+        <x:v>annotations/073_trigone_atrium_of_the_lateral_ventricle.nii.gz</x:v>
+      </x:c>
       <x:c r="J106" s="35" t="str"/>
       <x:c r="K106" s="35" t="str"/>
       <x:c r="L106" s="36" t="str"/>
     </x:row>
     <x:row r="107">
-      <x:c r="A107" s="37" t="str">
-        <x:v>yes</x:v>
-      </x:c>
-      <x:c r="B107" s="38" t="str">
-        <x:v>advanced</x:v>
-      </x:c>
-      <x:c r="C107" s="39" t="str">
+      <x:c r="A107" s="33" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="B107" s="34" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="C107" s="35" t="str">
+        <x:v>uncus</x:v>
+      </x:c>
+      <x:c r="D107" s="35" t="str">
+        <x:v>Uncus</x:v>
+      </x:c>
+      <x:c r="E107" s="35" t="str">
+        <x:v>limbic; cortex</x:v>
+      </x:c>
+      <x:c r="F107" s="35" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="G107" s="35" t="str"/>
+      <x:c r="H107" s="35" t="str"/>
+      <x:c r="I107" s="35" t="str"/>
+      <x:c r="J107" s="35" t="str"/>
+      <x:c r="K107" s="35" t="str"/>
+      <x:c r="L107" s="36" t="str"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="37" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="B108" s="38" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="C108" s="39" t="str">
         <x:v>vermis</x:v>
       </x:c>
-      <x:c r="D107" s="39" t="str">
+      <x:c r="D108" s="39" t="str">
         <x:v>Vermis</x:v>
       </x:c>
-      <x:c r="E107" s="39" t="str">
+      <x:c r="E108" s="39" t="str">
         <x:v>cerebellum; midline</x:v>
       </x:c>
-      <x:c r="F107" s="39" t="str">
+      <x:c r="F108" s="39" t="str">
         <x:v>no</x:v>
       </x:c>
-      <x:c r="G107" s="39" t="str"/>
-      <x:c r="H107" s="39" t="str"/>
-      <x:c r="I107" s="39" t="str"/>
-      <x:c r="J107" s="39" t="str"/>
-      <x:c r="K107" s="39" t="str"/>
-      <x:c r="L107" s="40" t="str"/>
+      <x:c r="G108" s="39" t="str"/>
+      <x:c r="H108" s="39" t="str"/>
+      <x:c r="I108" s="39" t="str"/>
+      <x:c r="J108" s="39" t="str"/>
+      <x:c r="K108" s="39" t="str"/>
+      <x:c r="L108" s="40" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">
-    <x:dataValidation type="list" sqref="A2:A107">
+    <x:dataValidation type="list" sqref="A2:A108">
       <x:formula1>"yes,no"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="B2:B107">
+    <x:dataValidation type="list" sqref="B2:B108">
       <x:formula1>"beginner,advanced"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30dc6bc66f7c4a6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85a0d8b8c2b9454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4482,16 +4528,16 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="45" t="str">
-        <x:v>crista_galli</x:v>
+        <x:v>corpus_callosum</x:v>
       </x:c>
       <x:c r="B24" s="35" t="str">
-        <x:v>Crista galli</x:v>
+        <x:v>Corpus callosum</x:v>
       </x:c>
       <x:c r="C24" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D24" s="35" t="str">
-        <x:v>skull_base; midline</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E24" s="34" t="str"/>
       <x:c r="F24" s="34" t="str"/>
@@ -4505,16 +4551,16 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="45" t="str">
-        <x:v>cuneus</x:v>
+        <x:v>crista_galli</x:v>
       </x:c>
       <x:c r="B25" s="35" t="str">
-        <x:v>Cuneus</x:v>
+        <x:v>Crista galli</x:v>
       </x:c>
       <x:c r="C25" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D25" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; midline</x:v>
       </x:c>
       <x:c r="E25" s="34" t="str"/>
       <x:c r="F25" s="34" t="str"/>
@@ -4528,16 +4574,16 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="45" t="str">
-        <x:v>entorhinal_cortex</x:v>
+        <x:v>cuneus</x:v>
       </x:c>
       <x:c r="B26" s="35" t="str">
-        <x:v>Entorhinal cortex</x:v>
+        <x:v>Cuneus</x:v>
       </x:c>
       <x:c r="C26" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D26" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E26" s="34" t="str"/>
       <x:c r="F26" s="34" t="str"/>
@@ -4551,16 +4597,16 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="45" t="str">
-        <x:v>external_auditory_canal</x:v>
+        <x:v>entorhinal_cortex</x:v>
       </x:c>
       <x:c r="B27" s="35" t="str">
-        <x:v>External auditory canal</x:v>
+        <x:v>Entorhinal cortex</x:v>
       </x:c>
       <x:c r="C27" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D27" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="E27" s="34" t="str"/>
       <x:c r="F27" s="34" t="str"/>
@@ -4574,16 +4620,16 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="45" t="str">
-        <x:v>falx_cerebri</x:v>
+        <x:v>external_auditory_canal</x:v>
       </x:c>
       <x:c r="B28" s="35" t="str">
-        <x:v>Falx cerebri</x:v>
+        <x:v>External auditory canal</x:v>
       </x:c>
       <x:c r="C28" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D28" s="35" t="str">
-        <x:v>midline</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="E28" s="34" t="str"/>
       <x:c r="F28" s="34" t="str"/>
@@ -4597,16 +4643,16 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="45" t="str">
-        <x:v>foramen_magnum</x:v>
+        <x:v>falx_cerebri</x:v>
       </x:c>
       <x:c r="B29" s="35" t="str">
-        <x:v>Foramen magnum</x:v>
+        <x:v>Falx cerebri</x:v>
       </x:c>
       <x:c r="C29" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D29" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>midline</x:v>
       </x:c>
       <x:c r="E29" s="34" t="str"/>
       <x:c r="F29" s="34" t="str"/>
@@ -4620,16 +4666,16 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="45" t="str">
-        <x:v>foramen_of_luschka</x:v>
+        <x:v>foramen_magnum</x:v>
       </x:c>
       <x:c r="B30" s="35" t="str">
-        <x:v>Foramen of Luschka</x:v>
+        <x:v>Foramen magnum</x:v>
       </x:c>
       <x:c r="C30" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D30" s="35" t="str">
-        <x:v>ventricles; csf_spaces; brainstem</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="E30" s="34" t="str"/>
       <x:c r="F30" s="34" t="str"/>
@@ -4643,10 +4689,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="45" t="str">
-        <x:v>foramen_of_magendie</x:v>
+        <x:v>foramen_of_luschka</x:v>
       </x:c>
       <x:c r="B31" s="35" t="str">
-        <x:v>Foramen of Magendie</x:v>
+        <x:v>Foramen of Luschka</x:v>
       </x:c>
       <x:c r="C31" s="35" t="str">
         <x:v>advanced</x:v>
@@ -4666,16 +4712,16 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="45" t="str">
-        <x:v>forceps_major</x:v>
+        <x:v>foramen_of_magendie</x:v>
       </x:c>
       <x:c r="B32" s="35" t="str">
-        <x:v>Forceps major</x:v>
+        <x:v>Foramen of Magendie</x:v>
       </x:c>
       <x:c r="C32" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D32" s="35" t="str">
-        <x:v>white_matter</x:v>
+        <x:v>ventricles; csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E32" s="34" t="str"/>
       <x:c r="F32" s="34" t="str"/>
@@ -4689,10 +4735,10 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="45" t="str">
-        <x:v>forceps_minor</x:v>
+        <x:v>forceps_major</x:v>
       </x:c>
       <x:c r="B33" s="35" t="str">
-        <x:v>Forceps minor</x:v>
+        <x:v>Forceps major</x:v>
       </x:c>
       <x:c r="C33" s="35" t="str">
         <x:v>advanced</x:v>
@@ -4712,16 +4758,16 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="45" t="str">
-        <x:v>fourth_ventricle</x:v>
+        <x:v>forceps_minor</x:v>
       </x:c>
       <x:c r="B34" s="35" t="str">
-        <x:v>Fourth ventricle</x:v>
+        <x:v>Forceps minor</x:v>
       </x:c>
       <x:c r="C34" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D34" s="35" t="str">
-        <x:v>ventricles; csf_spaces; brainstem</x:v>
+        <x:v>white_matter</x:v>
       </x:c>
       <x:c r="E34" s="34" t="str"/>
       <x:c r="F34" s="34" t="str"/>
@@ -4735,16 +4781,16 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="45" t="str">
-        <x:v>frontal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>fourth_ventricle</x:v>
       </x:c>
       <x:c r="B35" s="35" t="str">
-        <x:v>Frontal horn of the lateral ventricle</x:v>
+        <x:v>Fourth ventricle</x:v>
       </x:c>
       <x:c r="C35" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D35" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E35" s="34" t="str"/>
       <x:c r="F35" s="34" t="str"/>
@@ -4758,16 +4804,16 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="45" t="str">
-        <x:v>frontal_lobe</x:v>
+        <x:v>frontal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B36" s="35" t="str">
-        <x:v>Frontal lobe</x:v>
+        <x:v>Frontal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C36" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D36" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E36" s="34" t="str"/>
       <x:c r="F36" s="34" t="str"/>
@@ -4781,16 +4827,16 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="45" t="str">
-        <x:v>fusiform_gyrus</x:v>
+        <x:v>frontal_lobe</x:v>
       </x:c>
       <x:c r="B37" s="35" t="str">
-        <x:v>Fusiform gyrus</x:v>
+        <x:v>Frontal lobe</x:v>
       </x:c>
       <x:c r="C37" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D37" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="E37" s="34" t="str"/>
       <x:c r="F37" s="34" t="str"/>
@@ -4804,16 +4850,16 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="45" t="str">
-        <x:v>genu_of_the_corpus_callosum</x:v>
+        <x:v>fusiform_gyrus</x:v>
       </x:c>
       <x:c r="B38" s="35" t="str">
-        <x:v>Genu of the corpus callosum</x:v>
+        <x:v>Fusiform gyrus</x:v>
       </x:c>
       <x:c r="C38" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D38" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E38" s="34" t="str"/>
       <x:c r="F38" s="34" t="str"/>
@@ -4827,16 +4873,16 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="45" t="str">
-        <x:v>genu_of_the_internal_capsule</x:v>
+        <x:v>genu_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="B39" s="35" t="str">
-        <x:v>Genu of the internal capsule</x:v>
+        <x:v>Genu of the corpus callosum</x:v>
       </x:c>
       <x:c r="C39" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D39" s="35" t="str">
-        <x:v>white_matter; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E39" s="34" t="str"/>
       <x:c r="F39" s="34" t="str"/>
@@ -4850,16 +4896,16 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="45" t="str">
-        <x:v>globus_pallidus</x:v>
+        <x:v>genu_of_the_internal_capsule</x:v>
       </x:c>
       <x:c r="B40" s="35" t="str">
-        <x:v>Globus pallidus</x:v>
+        <x:v>Genu of the internal capsule</x:v>
       </x:c>
       <x:c r="C40" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D40" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>white_matter; basal_ganglia</x:v>
       </x:c>
       <x:c r="E40" s="34" t="str"/>
       <x:c r="F40" s="34" t="str"/>
@@ -4873,16 +4919,16 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="45" t="str">
-        <x:v>gyrus_rectus</x:v>
+        <x:v>globus_pallidus</x:v>
       </x:c>
       <x:c r="B41" s="35" t="str">
-        <x:v>Gyrus rectus</x:v>
+        <x:v>Globus pallidus</x:v>
       </x:c>
       <x:c r="C41" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D41" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="E41" s="34" t="str"/>
       <x:c r="F41" s="34" t="str"/>
@@ -4896,16 +4942,16 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="45" t="str">
-        <x:v>habenula</x:v>
+        <x:v>gyrus_rectus</x:v>
       </x:c>
       <x:c r="B42" s="35" t="str">
-        <x:v>Habenula</x:v>
+        <x:v>Gyrus rectus</x:v>
       </x:c>
       <x:c r="C42" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D42" s="35" t="str">
-        <x:v>midline; deep_gray</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E42" s="34" t="str"/>
       <x:c r="F42" s="34" t="str"/>
@@ -4919,16 +4965,16 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="45" t="str">
-        <x:v>hand_bump_of_the_precentral_gyrus</x:v>
+        <x:v>habenula</x:v>
       </x:c>
       <x:c r="B43" s="35" t="str">
-        <x:v>Hand bump of the precentral gyrus</x:v>
+        <x:v>Habenula</x:v>
       </x:c>
       <x:c r="C43" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D43" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>midline; deep_gray</x:v>
       </x:c>
       <x:c r="E43" s="34" t="str"/>
       <x:c r="F43" s="34" t="str"/>
@@ -4942,16 +4988,16 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="45" t="str">
-        <x:v>head_of_the_caudate_nucleus</x:v>
+        <x:v>hand_bump_of_the_precentral_gyrus</x:v>
       </x:c>
       <x:c r="B44" s="35" t="str">
-        <x:v>Head of the caudate nucleus</x:v>
+        <x:v>Hand bump of the precentral gyrus</x:v>
       </x:c>
       <x:c r="C44" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D44" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E44" s="34" t="str"/>
       <x:c r="F44" s="34" t="str"/>
@@ -4965,16 +5011,16 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="45" t="str">
-        <x:v>hippocampus</x:v>
+        <x:v>head_of_the_caudate_nucleus</x:v>
       </x:c>
       <x:c r="B45" s="35" t="str">
-        <x:v>Hippocampus</x:v>
+        <x:v>Head of the caudate nucleus</x:v>
       </x:c>
       <x:c r="C45" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D45" s="35" t="str">
-        <x:v>limbic</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="E45" s="34" t="str"/>
       <x:c r="F45" s="34" t="str"/>
@@ -4988,16 +5034,16 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="45" t="str">
-        <x:v>inferior_colliculus</x:v>
+        <x:v>hippocampus</x:v>
       </x:c>
       <x:c r="B46" s="35" t="str">
-        <x:v>Inferior colliculus</x:v>
+        <x:v>Hippocampus</x:v>
       </x:c>
       <x:c r="C46" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D46" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>limbic</x:v>
       </x:c>
       <x:c r="E46" s="34" t="str"/>
       <x:c r="F46" s="34" t="str"/>
@@ -5011,16 +5057,16 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="45" t="str">
-        <x:v>inferior_temporal_gyrus</x:v>
+        <x:v>inferior_colliculus</x:v>
       </x:c>
       <x:c r="B47" s="35" t="str">
-        <x:v>Inferior temporal gyrus</x:v>
+        <x:v>Inferior colliculus</x:v>
       </x:c>
       <x:c r="C47" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D47" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="E47" s="34" t="str"/>
       <x:c r="F47" s="34" t="str"/>
@@ -5034,13 +5080,13 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="45" t="str">
-        <x:v>insular_cortex</x:v>
+        <x:v>inferior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="B48" s="35" t="str">
-        <x:v>Insular cortex</x:v>
+        <x:v>Inferior temporal gyrus</x:v>
       </x:c>
       <x:c r="C48" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D48" s="35" t="str">
         <x:v>cortex</x:v>
@@ -5057,16 +5103,16 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="45" t="str">
-        <x:v>internal_auditory_canal</x:v>
+        <x:v>insular_cortex</x:v>
       </x:c>
       <x:c r="B49" s="35" t="str">
-        <x:v>Internal auditory canal</x:v>
+        <x:v>Insular cortex</x:v>
       </x:c>
       <x:c r="C49" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D49" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E49" s="34" t="str"/>
       <x:c r="F49" s="34" t="str"/>
@@ -5080,16 +5126,16 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="45" t="str">
-        <x:v>interpeduncular_cistern</x:v>
+        <x:v>internal_auditory_canal</x:v>
       </x:c>
       <x:c r="B50" s="35" t="str">
-        <x:v>Interpeduncular cistern</x:v>
+        <x:v>Internal auditory canal</x:v>
       </x:c>
       <x:c r="C50" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D50" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="E50" s="34" t="str"/>
       <x:c r="F50" s="34" t="str"/>
@@ -5103,16 +5149,16 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="45" t="str">
-        <x:v>interventricular_foramen_foramen_of_monro</x:v>
+        <x:v>interpeduncular_cistern</x:v>
       </x:c>
       <x:c r="B51" s="35" t="str">
-        <x:v>Interventricular foramen (foramen of Monro)</x:v>
+        <x:v>Interpeduncular cistern</x:v>
       </x:c>
       <x:c r="C51" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D51" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E51" s="34" t="str"/>
       <x:c r="F51" s="34" t="str"/>
@@ -5126,16 +5172,16 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="45" t="str">
-        <x:v>lateral_ventricle</x:v>
+        <x:v>interventricular_foramen_foramen_of_monro</x:v>
       </x:c>
       <x:c r="B52" s="35" t="str">
-        <x:v>Lateral Ventricle</x:v>
+        <x:v>Interventricular foramen (foramen of Monro)</x:v>
       </x:c>
       <x:c r="C52" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D52" s="35" t="str">
-        <x:v>csf_spaces; ventricles</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E52" s="34" t="str"/>
       <x:c r="F52" s="34" t="str"/>
@@ -5149,16 +5195,16 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="45" t="str">
-        <x:v>lentiform_nucleus</x:v>
+        <x:v>lateral_ventricle</x:v>
       </x:c>
       <x:c r="B53" s="35" t="str">
-        <x:v>Lentiform nucleus</x:v>
+        <x:v>Lateral Ventricle</x:v>
       </x:c>
       <x:c r="C53" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D53" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>csf_spaces; ventricles</x:v>
       </x:c>
       <x:c r="E53" s="34" t="str"/>
       <x:c r="F53" s="34" t="str"/>
@@ -5172,16 +5218,16 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="45" t="str">
-        <x:v>lingual_gyrus</x:v>
+        <x:v>lentiform_nucleus</x:v>
       </x:c>
       <x:c r="B54" s="35" t="str">
-        <x:v>Lingual gyrus</x:v>
+        <x:v>Lentiform nucleus</x:v>
       </x:c>
       <x:c r="C54" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D54" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="E54" s="34" t="str"/>
       <x:c r="F54" s="34" t="str"/>
@@ -5195,16 +5241,16 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="45" t="str">
-        <x:v>mammillary_bodies</x:v>
+        <x:v>lingual_gyrus</x:v>
       </x:c>
       <x:c r="B55" s="35" t="str">
-        <x:v>Mammillary bodies</x:v>
+        <x:v>Lingual gyrus</x:v>
       </x:c>
       <x:c r="C55" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D55" s="35" t="str">
-        <x:v>limbic; midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E55" s="34" t="str"/>
       <x:c r="F55" s="34" t="str"/>
@@ -5218,16 +5264,16 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="45" t="str">
-        <x:v>marginal_sulcus_pars_marginalis</x:v>
+        <x:v>mammillary_bodies</x:v>
       </x:c>
       <x:c r="B56" s="35" t="str">
-        <x:v>Marginal sulcus (pars marginalis)</x:v>
+        <x:v>Mammillary bodies</x:v>
       </x:c>
       <x:c r="C56" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D56" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>limbic; midline</x:v>
       </x:c>
       <x:c r="E56" s="34" t="str"/>
       <x:c r="F56" s="34" t="str"/>
@@ -5241,16 +5287,16 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="45" t="str">
-        <x:v>meckel_s_cave</x:v>
+        <x:v>marginal_sulcus_pars_marginalis</x:v>
       </x:c>
       <x:c r="B57" s="35" t="str">
-        <x:v>Meckel's cave</x:v>
+        <x:v>Marginal sulcus (pars marginalis)</x:v>
       </x:c>
       <x:c r="C57" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D57" s="35" t="str">
-        <x:v>skull_base; cranial_nerves; csf_spaces</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="E57" s="34" t="str"/>
       <x:c r="F57" s="34" t="str"/>
@@ -5264,16 +5310,16 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="45" t="str">
-        <x:v>median_interhemispheric_fissure</x:v>
+        <x:v>meckel_s_cave</x:v>
       </x:c>
       <x:c r="B58" s="35" t="str">
-        <x:v>Median interhemispheric fissure</x:v>
+        <x:v>Meckel's cave</x:v>
       </x:c>
       <x:c r="C58" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D58" s="35" t="str">
-        <x:v>csf_spaces; midline</x:v>
+        <x:v>skull_base; cranial_nerves; csf_spaces</x:v>
       </x:c>
       <x:c r="E58" s="34" t="str"/>
       <x:c r="F58" s="34" t="str"/>
@@ -5287,16 +5333,16 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="45" t="str">
-        <x:v>medulla_oblongata</x:v>
+        <x:v>median_interhemispheric_fissure</x:v>
       </x:c>
       <x:c r="B59" s="35" t="str">
-        <x:v>Medulla oblongata</x:v>
+        <x:v>Median interhemispheric fissure</x:v>
       </x:c>
       <x:c r="C59" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D59" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>csf_spaces; midline</x:v>
       </x:c>
       <x:c r="E59" s="34" t="str"/>
       <x:c r="F59" s="34" t="str"/>
@@ -5310,10 +5356,10 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="45" t="str">
-        <x:v>midbrain</x:v>
+        <x:v>medulla_oblongata</x:v>
       </x:c>
       <x:c r="B60" s="35" t="str">
-        <x:v>Midbrain</x:v>
+        <x:v>Medulla oblongata</x:v>
       </x:c>
       <x:c r="C60" s="35" t="str">
         <x:v>beginner</x:v>
@@ -5333,16 +5379,16 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="45" t="str">
-        <x:v>middle_cerebellar_peduncle</x:v>
+        <x:v>midbrain</x:v>
       </x:c>
       <x:c r="B61" s="35" t="str">
-        <x:v>Middle cerebellar peduncle</x:v>
+        <x:v>Midbrain</x:v>
       </x:c>
       <x:c r="C61" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D61" s="35" t="str">
-        <x:v>white_matter; cerebellum; brainstem</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="E61" s="34" t="str"/>
       <x:c r="F61" s="34" t="str"/>
@@ -5356,16 +5402,16 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="45" t="str">
-        <x:v>middle_temporal_gyrus</x:v>
+        <x:v>middle_cerebellar_peduncle</x:v>
       </x:c>
       <x:c r="B62" s="35" t="str">
-        <x:v>Middle temporal gyrus</x:v>
+        <x:v>Middle cerebellar peduncle</x:v>
       </x:c>
       <x:c r="C62" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D62" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>white_matter; cerebellum; brainstem</x:v>
       </x:c>
       <x:c r="E62" s="34" t="str"/>
       <x:c r="F62" s="34" t="str"/>
@@ -5379,16 +5425,16 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="45" t="str">
-        <x:v>nodule_of_the_cerebellum</x:v>
+        <x:v>middle_temporal_gyrus</x:v>
       </x:c>
       <x:c r="B63" s="35" t="str">
-        <x:v>Nodule of the cerebellum</x:v>
+        <x:v>Middle temporal gyrus</x:v>
       </x:c>
       <x:c r="C63" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D63" s="35" t="str">
-        <x:v>cerebellum; midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E63" s="34" t="str"/>
       <x:c r="F63" s="34" t="str"/>
@@ -5402,16 +5448,16 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="45" t="str">
-        <x:v>nucleus_accumbens</x:v>
+        <x:v>nodule_of_the_cerebellum</x:v>
       </x:c>
       <x:c r="B64" s="35" t="str">
-        <x:v>Nucleus accumbens</x:v>
+        <x:v>Nodule of the cerebellum</x:v>
       </x:c>
       <x:c r="C64" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D64" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>cerebellum; midline</x:v>
       </x:c>
       <x:c r="E64" s="34" t="str"/>
       <x:c r="F64" s="34" t="str"/>
@@ -5425,16 +5471,16 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="45" t="str">
-        <x:v>occipital_horn_of_the_lateral_ventricle</x:v>
+        <x:v>nucleus_accumbens</x:v>
       </x:c>
       <x:c r="B65" s="35" t="str">
-        <x:v>Occipital horn of the lateral ventricle</x:v>
+        <x:v>Nucleus accumbens</x:v>
       </x:c>
       <x:c r="C65" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D65" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="E65" s="34" t="str"/>
       <x:c r="F65" s="34" t="str"/>
@@ -5448,16 +5494,16 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="45" t="str">
-        <x:v>occipital_lobe</x:v>
+        <x:v>occipital_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B66" s="35" t="str">
-        <x:v>Occipital lobe</x:v>
+        <x:v>Occipital horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C66" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D66" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E66" s="34" t="str"/>
       <x:c r="F66" s="34" t="str"/>
@@ -5471,16 +5517,16 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="45" t="str">
-        <x:v>optic_chiasm</x:v>
+        <x:v>occipital_lobe</x:v>
       </x:c>
       <x:c r="B67" s="35" t="str">
-        <x:v>Optic chiasm</x:v>
+        <x:v>Occipital lobe</x:v>
       </x:c>
       <x:c r="C67" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D67" s="35" t="str">
-        <x:v>cranial_nerves; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E67" s="34" t="str"/>
       <x:c r="F67" s="34" t="str"/>
@@ -5494,16 +5540,16 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="45" t="str">
-        <x:v>optic_nerve</x:v>
+        <x:v>optic_chiasm</x:v>
       </x:c>
       <x:c r="B68" s="35" t="str">
-        <x:v>Optic nerve</x:v>
+        <x:v>Optic chiasm</x:v>
       </x:c>
       <x:c r="C68" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D68" s="35" t="str">
-        <x:v>cranial_nerves; skull_base; orbit</x:v>
+        <x:v>cranial_nerves; skull_base</x:v>
       </x:c>
       <x:c r="E68" s="34" t="str"/>
       <x:c r="F68" s="34" t="str"/>
@@ -5517,16 +5563,16 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="45" t="str">
-        <x:v>orbitofrontal_cortex</x:v>
+        <x:v>optic_nerve</x:v>
       </x:c>
       <x:c r="B69" s="35" t="str">
-        <x:v>Orbitofrontal cortex</x:v>
+        <x:v>Optic nerve</x:v>
       </x:c>
       <x:c r="C69" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D69" s="35" t="str">
-        <x:v>cortex; skull_base</x:v>
+        <x:v>cranial_nerves; skull_base; orbit</x:v>
       </x:c>
       <x:c r="E69" s="34" t="str"/>
       <x:c r="F69" s="34" t="str"/>
@@ -5540,16 +5586,16 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="45" t="str">
-        <x:v>parahippocampal_gyrus</x:v>
+        <x:v>orbitofrontal_cortex</x:v>
       </x:c>
       <x:c r="B70" s="35" t="str">
-        <x:v>Parahippocampal gyrus</x:v>
+        <x:v>Orbitofrontal cortex</x:v>
       </x:c>
       <x:c r="C70" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D70" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex; skull_base</x:v>
       </x:c>
       <x:c r="E70" s="34" t="str"/>
       <x:c r="F70" s="34" t="str"/>
@@ -5563,16 +5609,16 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="45" t="str">
-        <x:v>parietal_lobe</x:v>
+        <x:v>parahippocampal_gyrus</x:v>
       </x:c>
       <x:c r="B71" s="35" t="str">
-        <x:v>Parietal lobe</x:v>
+        <x:v>Parahippocampal gyrus</x:v>
       </x:c>
       <x:c r="C71" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D71" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="E71" s="34" t="str"/>
       <x:c r="F71" s="34" t="str"/>
@@ -5586,16 +5632,16 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="45" t="str">
-        <x:v>parieto_occipital_sulcus</x:v>
+        <x:v>parietal_lobe</x:v>
       </x:c>
       <x:c r="B72" s="35" t="str">
-        <x:v>Parieto-occipital sulcus</x:v>
+        <x:v>Parietal lobe</x:v>
       </x:c>
       <x:c r="C72" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D72" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="E72" s="34" t="str"/>
       <x:c r="F72" s="34" t="str"/>
@@ -5609,10 +5655,10 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="45" t="str">
-        <x:v>pars_opercularis</x:v>
+        <x:v>parieto_occipital_sulcus</x:v>
       </x:c>
       <x:c r="B73" s="35" t="str">
-        <x:v>Pars opercularis</x:v>
+        <x:v>Parieto-occipital sulcus</x:v>
       </x:c>
       <x:c r="C73" s="35" t="str">
         <x:v>advanced</x:v>
@@ -5632,10 +5678,10 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="45" t="str">
-        <x:v>pars_orbitalis</x:v>
+        <x:v>pars_opercularis</x:v>
       </x:c>
       <x:c r="B74" s="35" t="str">
-        <x:v>Pars orbitalis</x:v>
+        <x:v>Pars opercularis</x:v>
       </x:c>
       <x:c r="C74" s="35" t="str">
         <x:v>advanced</x:v>
@@ -5655,10 +5701,10 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="45" t="str">
-        <x:v>pars_triangularis</x:v>
+        <x:v>pars_orbitalis</x:v>
       </x:c>
       <x:c r="B75" s="35" t="str">
-        <x:v>Pars triangularis</x:v>
+        <x:v>Pars orbitalis</x:v>
       </x:c>
       <x:c r="C75" s="35" t="str">
         <x:v>advanced</x:v>
@@ -5678,16 +5724,16 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="45" t="str">
-        <x:v>pineal_gland</x:v>
+        <x:v>pars_triangularis</x:v>
       </x:c>
       <x:c r="B76" s="35" t="str">
-        <x:v>Pineal gland</x:v>
+        <x:v>Pars triangularis</x:v>
       </x:c>
       <x:c r="C76" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D76" s="35" t="str">
-        <x:v>midline</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E76" s="34" t="str"/>
       <x:c r="F76" s="34" t="str"/>
@@ -5701,16 +5747,16 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="45" t="str">
-        <x:v>pituitary_fossa</x:v>
+        <x:v>pineal_gland</x:v>
       </x:c>
       <x:c r="B77" s="35" t="str">
-        <x:v>Pituitary fossa</x:v>
+        <x:v>Pineal gland</x:v>
       </x:c>
       <x:c r="C77" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D77" s="35" t="str">
-        <x:v>skull_base; midline</x:v>
+        <x:v>midline</x:v>
       </x:c>
       <x:c r="E77" s="34" t="str"/>
       <x:c r="F77" s="34" t="str"/>
@@ -5724,16 +5770,16 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="45" t="str">
-        <x:v>pons</x:v>
+        <x:v>pituitary_fossa</x:v>
       </x:c>
       <x:c r="B78" s="35" t="str">
-        <x:v>Pons</x:v>
+        <x:v>Pituitary fossa</x:v>
       </x:c>
       <x:c r="C78" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D78" s="35" t="str">
-        <x:v>brainstem</x:v>
+        <x:v>skull_base; midline</x:v>
       </x:c>
       <x:c r="E78" s="34" t="str"/>
       <x:c r="F78" s="34" t="str"/>
@@ -5747,16 +5793,16 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="45" t="str">
-        <x:v>postcentral_gyrus</x:v>
+        <x:v>pons</x:v>
       </x:c>
       <x:c r="B79" s="35" t="str">
-        <x:v>Postcentral gyrus</x:v>
+        <x:v>Pons</x:v>
       </x:c>
       <x:c r="C79" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D79" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>brainstem</x:v>
       </x:c>
       <x:c r="E79" s="34" t="str"/>
       <x:c r="F79" s="34" t="str"/>
@@ -5770,16 +5816,16 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="45" t="str">
-        <x:v>posterior_cingulate_gyrus</x:v>
+        <x:v>postcentral_gyrus</x:v>
       </x:c>
       <x:c r="B80" s="35" t="str">
-        <x:v>Posterior cingulate gyrus</x:v>
+        <x:v>Postcentral gyrus</x:v>
       </x:c>
       <x:c r="C80" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D80" s="35" t="str">
-        <x:v>cortex; limbic</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E80" s="34" t="str"/>
       <x:c r="F80" s="34" t="str"/>
@@ -5793,16 +5839,16 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="45" t="str">
-        <x:v>posterior_commissure</x:v>
+        <x:v>posterior_cingulate_gyrus</x:v>
       </x:c>
       <x:c r="B81" s="35" t="str">
-        <x:v>Posterior commissure</x:v>
+        <x:v>Posterior cingulate gyrus</x:v>
       </x:c>
       <x:c r="C81" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D81" s="35" t="str">
-        <x:v>white_matter; midline; brainstem</x:v>
+        <x:v>cortex; limbic</x:v>
       </x:c>
       <x:c r="E81" s="34" t="str"/>
       <x:c r="F81" s="34" t="str"/>
@@ -5816,16 +5862,16 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="45" t="str">
-        <x:v>posterior_limb_of_the_internal_capsule</x:v>
+        <x:v>posterior_commissure</x:v>
       </x:c>
       <x:c r="B82" s="35" t="str">
-        <x:v>Posterior limb of the internal capsule</x:v>
+        <x:v>Posterior commissure</x:v>
       </x:c>
       <x:c r="C82" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D82" s="35" t="str">
-        <x:v>white_matter; basal_ganglia</x:v>
+        <x:v>white_matter; midline; brainstem</x:v>
       </x:c>
       <x:c r="E82" s="34" t="str"/>
       <x:c r="F82" s="34" t="str"/>
@@ -5839,16 +5885,16 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="45" t="str">
-        <x:v>precentral_gyrus</x:v>
+        <x:v>posterior_limb_of_the_internal_capsule</x:v>
       </x:c>
       <x:c r="B83" s="35" t="str">
-        <x:v>Precentral gyrus</x:v>
+        <x:v>Posterior limb of the internal capsule</x:v>
       </x:c>
       <x:c r="C83" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D83" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>white_matter; basal_ganglia</x:v>
       </x:c>
       <x:c r="E83" s="34" t="str"/>
       <x:c r="F83" s="34" t="str"/>
@@ -5862,13 +5908,13 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="45" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>precentral_gyrus</x:v>
       </x:c>
       <x:c r="B84" s="35" t="str">
-        <x:v>precuneus</x:v>
+        <x:v>Precentral gyrus</x:v>
       </x:c>
       <x:c r="C84" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D84" s="35" t="str">
         <x:v>cortex</x:v>
@@ -5885,16 +5931,16 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="45" t="str">
-        <x:v>premedullary_cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="B85" s="35" t="str">
-        <x:v>Premedullary cistern</x:v>
+        <x:v>precuneus</x:v>
       </x:c>
       <x:c r="C85" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D85" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E85" s="34" t="str"/>
       <x:c r="F85" s="34" t="str"/>
@@ -5908,10 +5954,10 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="45" t="str">
-        <x:v>prepontine_cistern</x:v>
+        <x:v>premedullary_cistern</x:v>
       </x:c>
       <x:c r="B86" s="35" t="str">
-        <x:v>Prepontine cistern</x:v>
+        <x:v>Premedullary cistern</x:v>
       </x:c>
       <x:c r="C86" s="35" t="str">
         <x:v>beginner</x:v>
@@ -5931,16 +5977,16 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="45" t="str">
-        <x:v>putamen</x:v>
+        <x:v>prepontine_cistern</x:v>
       </x:c>
       <x:c r="B87" s="35" t="str">
-        <x:v>Putamen</x:v>
+        <x:v>Prepontine cistern</x:v>
       </x:c>
       <x:c r="C87" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D87" s="35" t="str">
-        <x:v>basal_ganglia; deep_gray</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E87" s="34" t="str"/>
       <x:c r="F87" s="34" t="str"/>
@@ -5954,16 +6000,16 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="45" t="str">
-        <x:v>quadrigeminal_cistern</x:v>
+        <x:v>putamen</x:v>
       </x:c>
       <x:c r="B88" s="35" t="str">
-        <x:v>Quadrigeminal cistern</x:v>
+        <x:v>Putamen</x:v>
       </x:c>
       <x:c r="C88" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D88" s="35" t="str">
-        <x:v>csf_spaces; brainstem</x:v>
+        <x:v>basal_ganglia; deep_gray</x:v>
       </x:c>
       <x:c r="E88" s="34" t="str"/>
       <x:c r="F88" s="34" t="str"/>
@@ -5977,16 +6023,16 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="45" t="str">
-        <x:v>rostrum_of_the_corpus_callosum</x:v>
+        <x:v>quadrigeminal_cistern</x:v>
       </x:c>
       <x:c r="B89" s="35" t="str">
-        <x:v>Rostrum of the corpus callosum</x:v>
+        <x:v>Quadrigeminal cistern</x:v>
       </x:c>
       <x:c r="C89" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D89" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>csf_spaces; brainstem</x:v>
       </x:c>
       <x:c r="E89" s="34" t="str"/>
       <x:c r="F89" s="34" t="str"/>
@@ -6000,16 +6046,16 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="45" t="str">
-        <x:v>septum_pellucidum</x:v>
+        <x:v>rostrum_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="B90" s="35" t="str">
-        <x:v>Septum pellucidum</x:v>
+        <x:v>Rostrum of the corpus callosum</x:v>
       </x:c>
       <x:c r="C90" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D90" s="35" t="str">
-        <x:v>midline; ventricles; csf_spaces</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E90" s="34" t="str"/>
       <x:c r="F90" s="34" t="str"/>
@@ -6023,16 +6069,16 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="45" t="str">
-        <x:v>splenium_of_the_corpus_callosum</x:v>
+        <x:v>septum_pellucidum</x:v>
       </x:c>
       <x:c r="B91" s="35" t="str">
-        <x:v>Splenium of the corpus callosum</x:v>
+        <x:v>Septum pellucidum</x:v>
       </x:c>
       <x:c r="C91" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D91" s="35" t="str">
-        <x:v>white_matter; midline</x:v>
+        <x:v>midline; ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E91" s="34" t="str"/>
       <x:c r="F91" s="34" t="str"/>
@@ -6046,16 +6092,16 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="45" t="str">
-        <x:v>subthalamic_region</x:v>
+        <x:v>splenium_of_the_corpus_callosum</x:v>
       </x:c>
       <x:c r="B92" s="35" t="str">
-        <x:v>Subthalamic region</x:v>
+        <x:v>Splenium of the corpus callosum</x:v>
       </x:c>
       <x:c r="C92" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D92" s="35" t="str">
-        <x:v>deep_gray; basal_ganglia</x:v>
+        <x:v>white_matter; midline</x:v>
       </x:c>
       <x:c r="E92" s="34" t="str"/>
       <x:c r="F92" s="34" t="str"/>
@@ -6069,16 +6115,16 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="45" t="str">
-        <x:v>superior_frontal_gyrus</x:v>
+        <x:v>subthalamic_region</x:v>
       </x:c>
       <x:c r="B93" s="35" t="str">
-        <x:v>Superior frontal gyrus</x:v>
+        <x:v>Subthalamic region</x:v>
       </x:c>
       <x:c r="C93" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D93" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>deep_gray; basal_ganglia</x:v>
       </x:c>
       <x:c r="E93" s="34" t="str"/>
       <x:c r="F93" s="34" t="str"/>
@@ -6092,16 +6138,16 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="45" t="str">
-        <x:v>superior_orbital_fissure</x:v>
+        <x:v>superior_frontal_gyrus</x:v>
       </x:c>
       <x:c r="B94" s="35" t="str">
-        <x:v>Superior orbital fissure</x:v>
+        <x:v>Superior frontal gyrus</x:v>
       </x:c>
       <x:c r="C94" s="35" t="str">
         <x:v>advanced</x:v>
       </x:c>
       <x:c r="D94" s="35" t="str">
-        <x:v>skull_base; cranial_nerves</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E94" s="34" t="str"/>
       <x:c r="F94" s="34" t="str"/>
@@ -6115,16 +6161,16 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="45" t="str">
-        <x:v>superior_temporal_gyrus</x:v>
+        <x:v>superior_orbital_fissure</x:v>
       </x:c>
       <x:c r="B95" s="35" t="str">
-        <x:v>Superior temporal gyrus</x:v>
+        <x:v>Superior orbital fissure</x:v>
       </x:c>
       <x:c r="C95" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D95" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>skull_base; cranial_nerves</x:v>
       </x:c>
       <x:c r="E95" s="34" t="str"/>
       <x:c r="F95" s="34" t="str"/>
@@ -6138,13 +6184,13 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="45" t="str">
-        <x:v>supramarginal_gyrus</x:v>
+        <x:v>superior_temporal_gyrus</x:v>
       </x:c>
       <x:c r="B96" s="35" t="str">
-        <x:v>Supramarginal gyrus</x:v>
+        <x:v>Superior temporal gyrus</x:v>
       </x:c>
       <x:c r="C96" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D96" s="35" t="str">
         <x:v>cortex</x:v>
@@ -6161,16 +6207,16 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="45" t="str">
-        <x:v>suprasellar_cistern</x:v>
+        <x:v>supramarginal_gyrus</x:v>
       </x:c>
       <x:c r="B97" s="35" t="str">
-        <x:v>Suprasellar cistern</x:v>
+        <x:v>Supramarginal gyrus</x:v>
       </x:c>
       <x:c r="C97" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D97" s="35" t="str">
-        <x:v>csf_spaces; skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E97" s="34" t="str"/>
       <x:c r="F97" s="34" t="str"/>
@@ -6184,16 +6230,16 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="45" t="str">
-        <x:v>sylvian_fissure</x:v>
+        <x:v>suprasellar_cistern</x:v>
       </x:c>
       <x:c r="B98" s="35" t="str">
-        <x:v>Sylvian fissure</x:v>
+        <x:v>Suprasellar cistern</x:v>
       </x:c>
       <x:c r="C98" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D98" s="35" t="str">
-        <x:v>csf_spaces; cortex</x:v>
+        <x:v>csf_spaces; skull_base</x:v>
       </x:c>
       <x:c r="E98" s="34" t="str"/>
       <x:c r="F98" s="34" t="str"/>
@@ -6207,16 +6253,16 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="45" t="str">
-        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
+        <x:v>sylvian_fissure</x:v>
       </x:c>
       <x:c r="B99" s="35" t="str">
-        <x:v>Temporal horn of the lateral ventricle</x:v>
+        <x:v>Sylvian fissure</x:v>
       </x:c>
       <x:c r="C99" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D99" s="35" t="str">
-        <x:v>ventricles; csf_spaces; deep_gray</x:v>
+        <x:v>csf_spaces; cortex</x:v>
       </x:c>
       <x:c r="E99" s="34" t="str"/>
       <x:c r="F99" s="34" t="str"/>
@@ -6230,16 +6276,16 @@
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="45" t="str">
-        <x:v>temporal_lobe</x:v>
+        <x:v>temporal_horn_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B100" s="35" t="str">
-        <x:v>Temporal lobe</x:v>
+        <x:v>Temporal horn of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C100" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D100" s="35" t="str">
-        <x:v>lobes; cortex</x:v>
+        <x:v>ventricles; csf_spaces; deep_gray</x:v>
       </x:c>
       <x:c r="E100" s="34" t="str"/>
       <x:c r="F100" s="34" t="str"/>
@@ -6253,16 +6299,16 @@
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="45" t="str">
-        <x:v>temporal_pole</x:v>
+        <x:v>temporal_lobe</x:v>
       </x:c>
       <x:c r="B101" s="35" t="str">
-        <x:v>Temporal pole</x:v>
+        <x:v>Temporal lobe</x:v>
       </x:c>
       <x:c r="C101" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D101" s="35" t="str">
-        <x:v>cortex</x:v>
+        <x:v>lobes; cortex</x:v>
       </x:c>
       <x:c r="E101" s="34" t="str"/>
       <x:c r="F101" s="34" t="str"/>
@@ -6276,16 +6322,16 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="45" t="str">
-        <x:v>tentorium_cerebelli</x:v>
+        <x:v>temporal_pole</x:v>
       </x:c>
       <x:c r="B102" s="35" t="str">
-        <x:v>Tentorium cerebelli</x:v>
+        <x:v>Temporal pole</x:v>
       </x:c>
       <x:c r="C102" s="35" t="str">
-        <x:v>beginner</x:v>
+        <x:v>advanced</x:v>
       </x:c>
       <x:c r="D102" s="35" t="str">
-        <x:v>skull_base</x:v>
+        <x:v>cortex</x:v>
       </x:c>
       <x:c r="E102" s="34" t="str"/>
       <x:c r="F102" s="34" t="str"/>
@@ -6299,16 +6345,16 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="45" t="str">
-        <x:v>thalamus</x:v>
+        <x:v>tentorium_cerebelli</x:v>
       </x:c>
       <x:c r="B103" s="35" t="str">
-        <x:v>Thalamus</x:v>
+        <x:v>Tentorium cerebelli</x:v>
       </x:c>
       <x:c r="C103" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D103" s="35" t="str">
-        <x:v>deep_gray</x:v>
+        <x:v>skull_base</x:v>
       </x:c>
       <x:c r="E103" s="34" t="str"/>
       <x:c r="F103" s="34" t="str"/>
@@ -6322,16 +6368,16 @@
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="45" t="str">
-        <x:v>third_ventricle</x:v>
+        <x:v>thalamus</x:v>
       </x:c>
       <x:c r="B104" s="35" t="str">
-        <x:v>Third ventricle</x:v>
+        <x:v>Thalamus</x:v>
       </x:c>
       <x:c r="C104" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D104" s="35" t="str">
-        <x:v>ventricles; csf_spaces; midline</x:v>
+        <x:v>deep_gray</x:v>
       </x:c>
       <x:c r="E104" s="34" t="str"/>
       <x:c r="F104" s="34" t="str"/>
@@ -6345,16 +6391,16 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="45" t="str">
-        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
+        <x:v>third_ventricle</x:v>
       </x:c>
       <x:c r="B105" s="35" t="str">
-        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
+        <x:v>Third ventricle</x:v>
       </x:c>
       <x:c r="C105" s="35" t="str">
         <x:v>beginner</x:v>
       </x:c>
       <x:c r="D105" s="35" t="str">
-        <x:v>ventricles; csf_spaces</x:v>
+        <x:v>ventricles; csf_spaces; midline</x:v>
       </x:c>
       <x:c r="E105" s="34" t="str"/>
       <x:c r="F105" s="34" t="str"/>
@@ -6368,16 +6414,16 @@
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="45" t="str">
-        <x:v>uncus</x:v>
+        <x:v>trigone_atrium_of_the_lateral_ventricle</x:v>
       </x:c>
       <x:c r="B106" s="35" t="str">
-        <x:v>Uncus</x:v>
+        <x:v>Trigone (atrium) of the lateral ventricle</x:v>
       </x:c>
       <x:c r="C106" s="35" t="str">
-        <x:v>advanced</x:v>
+        <x:v>beginner</x:v>
       </x:c>
       <x:c r="D106" s="35" t="str">
-        <x:v>limbic; cortex</x:v>
+        <x:v>ventricles; csf_spaces</x:v>
       </x:c>
       <x:c r="E106" s="34" t="str"/>
       <x:c r="F106" s="34" t="str"/>
@@ -6390,32 +6436,55 @@
       <x:c r="M106" s="36" t="str"/>
     </x:row>
     <x:row r="107">
-      <x:c r="A107" s="46" t="str">
+      <x:c r="A107" s="45" t="str">
+        <x:v>uncus</x:v>
+      </x:c>
+      <x:c r="B107" s="35" t="str">
+        <x:v>Uncus</x:v>
+      </x:c>
+      <x:c r="C107" s="35" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="D107" s="35" t="str">
+        <x:v>limbic; cortex</x:v>
+      </x:c>
+      <x:c r="E107" s="34" t="str"/>
+      <x:c r="F107" s="34" t="str"/>
+      <x:c r="G107" s="34" t="str"/>
+      <x:c r="H107" s="34" t="str"/>
+      <x:c r="I107" s="34" t="str"/>
+      <x:c r="J107" s="34" t="str"/>
+      <x:c r="K107" s="34" t="str"/>
+      <x:c r="L107" s="34" t="str"/>
+      <x:c r="M107" s="36" t="str"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="46" t="str">
         <x:v>vermis</x:v>
       </x:c>
-      <x:c r="B107" s="39" t="str">
+      <x:c r="B108" s="39" t="str">
         <x:v>Vermis</x:v>
       </x:c>
-      <x:c r="C107" s="39" t="str">
-        <x:v>advanced</x:v>
-      </x:c>
-      <x:c r="D107" s="39" t="str">
+      <x:c r="C108" s="39" t="str">
+        <x:v>advanced</x:v>
+      </x:c>
+      <x:c r="D108" s="39" t="str">
         <x:v>cerebellum; midline</x:v>
       </x:c>
-      <x:c r="E107" s="38" t="str"/>
-      <x:c r="F107" s="38" t="str"/>
-      <x:c r="G107" s="38" t="str"/>
-      <x:c r="H107" s="38" t="str"/>
-      <x:c r="I107" s="38" t="str"/>
-      <x:c r="J107" s="38" t="str"/>
-      <x:c r="K107" s="38" t="str"/>
-      <x:c r="L107" s="38" t="str"/>
-      <x:c r="M107" s="40" t="str"/>
+      <x:c r="E108" s="38" t="str"/>
+      <x:c r="F108" s="38" t="str"/>
+      <x:c r="G108" s="38" t="str"/>
+      <x:c r="H108" s="38" t="str"/>
+      <x:c r="I108" s="38" t="str"/>
+      <x:c r="J108" s="38" t="str"/>
+      <x:c r="K108" s="38" t="str"/>
+      <x:c r="L108" s="38" t="str"/>
+      <x:c r="M108" s="40" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39c52bf375db4545"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374f9ab7d0ec4b1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rename insula and mammillary body labels
</commit_message>
<xml_diff>
--- a/data/finalized/curation/brain_mri_curation.xlsx
+++ b/data/finalized/curation/brain_mri_curation.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R14949da8a8db4248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="Rd337bb02575a4ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="Re6d25cd770dd46b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R9debc60cd6dd4307"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structures" sheetId="2" r:id="R6dc42048bf1d4e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz Questions" sheetId="3" r:id="Ra98a1655dbbd4a8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2171,7 +2171,7 @@
         <x:v>insular_cortex</x:v>
       </x:c>
       <x:c r="D49" s="35" t="str">
-        <x:v>Insular cortex</x:v>
+        <x:v>Insula</x:v>
       </x:c>
       <x:c r="E49" s="35" t="str">
         <x:v>cortex</x:v>
@@ -2186,7 +2186,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I49" s="35" t="str">
-        <x:v>annotations/027_insular_cortex.nii.gz</x:v>
+        <x:v>annotations/027_insula.nii.gz</x:v>
       </x:c>
       <x:c r="J49" s="35" t="str"/>
       <x:c r="K49" s="35" t="str"/>
@@ -2381,7 +2381,7 @@
         <x:v>mammillary_bodies</x:v>
       </x:c>
       <x:c r="D56" s="35" t="str">
-        <x:v>Mammillary bodies</x:v>
+        <x:v>Mammillary body</x:v>
       </x:c>
       <x:c r="E56" s="35" t="str">
         <x:v>limbic; midline</x:v>
@@ -2396,7 +2396,7 @@
         <x:v>accepted</x:v>
       </x:c>
       <x:c r="I56" s="35" t="str">
-        <x:v>annotations/052_mammillary_bodies.nii.gz</x:v>
+        <x:v>annotations/052_mammillary_body.nii.gz</x:v>
       </x:c>
       <x:c r="J56" s="35" t="str"/>
       <x:c r="K56" s="35" t="str"/>
@@ -3955,7 +3955,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85a0d8b8c2b9454e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7b02c318c8e45e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5106,7 +5106,7 @@
         <x:v>insular_cortex</x:v>
       </x:c>
       <x:c r="B49" s="35" t="str">
-        <x:v>Insular cortex</x:v>
+        <x:v>Insula</x:v>
       </x:c>
       <x:c r="C49" s="35" t="str">
         <x:v>beginner</x:v>
@@ -5267,7 +5267,7 @@
         <x:v>mammillary_bodies</x:v>
       </x:c>
       <x:c r="B56" s="35" t="str">
-        <x:v>Mammillary bodies</x:v>
+        <x:v>Mammillary body</x:v>
       </x:c>
       <x:c r="C56" s="35" t="str">
         <x:v>beginner</x:v>
@@ -6484,7 +6484,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R374f9ab7d0ec4b1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44a72a788ee34b3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>